<commit_message>
docs(atlas): bound Shopping List XLSX print rhythm
</commit_message>
<xml_diff>
--- a/docs/xlsx/examples/atlas-shopping-list-v1-example.xlsx
+++ b/docs/xlsx/examples/atlas-shopping-list-v1-example.xlsx
@@ -26,25 +26,36 @@
     <numFmt numFmtId="200" formatCode="0.######"/>
     <numFmt numFmtId="201" formatCode="0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
     </font>
     <font>
-      <sz val="15"/>
+      <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
-      <sz val="20"/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
-      <sz val="15"/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
     </font>
@@ -66,7 +77,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="13">
     <border/>
     <border>
       <left style="thin">
@@ -93,6 +104,104 @@
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
     </border>
@@ -142,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -157,73 +266,127 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="0"/>
     </xf>
     <xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
     </xf>
     <xf numFmtId="200" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="200" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="201" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="200" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="200" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="201" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="201" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -268,6 +431,14 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -276,35 +447,51 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -317,26 +504,26 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="200" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -349,105 +536,225 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="200" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="201" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="200" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="200" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="201" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="201" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -707,15 +1014,15 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17.5" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="35" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="7.5" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="39" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="6.5" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="10.5" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="23" hidden="0" customWidth="1"/>
     <col min="6" max="17" width="1" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1" ht="29" customHeight="1">
       <c r="A1" s="4" t="str">
         <v>Thứ Hai (20/04/2026)</v>
       </c>
@@ -736,7 +1043,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="9" customHeight="1">
+    <row r="2" ht="5" customHeight="1">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -755,20 +1062,20 @@
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
     </row>
-    <row r="3" ht="39" customHeight="1">
-      <c r="A3" s="25" t="str">
+    <row r="3" ht="29" customHeight="1">
+      <c r="A3" s="42" t="str">
         <v>TRƯỜNG</v>
       </c>
-      <c r="B3" s="26" t="str">
+      <c r="B3" s="43" t="str">
         <v>THÀNH PHẦN</v>
       </c>
-      <c r="C3" s="26" t="str">
+      <c r="C3" s="43" t="str">
         <v>ĐVT</v>
       </c>
-      <c r="D3" s="26" t="str">
+      <c r="D3" s="43" t="str">
         <v>SỐ LƯỢNG</v>
       </c>
-      <c r="E3" s="27" t="str">
+      <c r="E3" s="44" t="str">
         <v>GHI CHÚ</v>
       </c>
       <c r="F3" s="2" t="str">
@@ -808,20 +1115,20 @@
         <v>__exported_note</v>
       </c>
     </row>
-    <row r="4" ht="96" customHeight="1">
-      <c r="A4" s="19" t="str">
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="28" t="str">
         <v>Trường Nguyễn Du - Cơ sở phía Đông</v>
       </c>
-      <c r="B4" s="15" t="str">
+      <c r="B4" s="18" t="str">
         <v>Ớt hiểm đỏ</v>
       </c>
-      <c r="C4" s="16" t="str">
+      <c r="C4" s="19" t="str">
         <v>Kg</v>
       </c>
-      <c r="D4" s="63" t="n">
+      <c r="D4" s="87" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="65" t="str">
+      <c r="E4" s="105" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -885,18 +1192,18 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="11" t="str"/>
-      <c r="B5" s="11" t="str">
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="30" t="str"/>
+      <c r="B5" s="14" t="str">
         <v>Tỏi</v>
       </c>
-      <c r="C5" s="12" t="str">
+      <c r="C5" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D5" s="69" t="n">
+      <c r="D5" s="93" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="57" t="str">
+      <c r="E5" s="109" t="str">
         <v>An Phú</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -960,18 +1267,18 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="11" t="str"/>
-      <c r="B6" s="11" t="str">
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="30" t="str"/>
+      <c r="B6" s="14" t="str">
         <v>Cà rốt</v>
       </c>
-      <c r="C6" s="12" t="str">
+      <c r="C6" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D6" s="69" t="n">
+      <c r="D6" s="93" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="57" t="str">
+      <c r="E6" s="109" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1035,18 +1342,18 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="11" t="str"/>
-      <c r="B7" s="11" t="str">
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="30" t="str"/>
+      <c r="B7" s="14" t="str">
         <v>Cải ngọt</v>
       </c>
-      <c r="C7" s="12" t="str">
+      <c r="C7" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D7" s="69" t="n">
+      <c r="D7" s="93" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="57" t="str">
+      <c r="E7" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1110,18 +1417,18 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="11" t="str"/>
-      <c r="B8" s="11" t="str">
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="30" t="str"/>
+      <c r="B8" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
       </c>
-      <c r="C8" s="12" t="str">
+      <c r="C8" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D8" s="55" t="n">
+      <c r="D8" s="79" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E8" s="57" t="str">
+      <c r="E8" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1185,18 +1492,18 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="11" t="str"/>
-      <c r="B9" s="11" t="str">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="30" t="str"/>
+      <c r="B9" s="14" t="str">
         <v>Hành lá</v>
       </c>
-      <c r="C9" s="12" t="str">
+      <c r="C9" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D9" s="55" t="n">
+      <c r="D9" s="79" t="n">
         <v>0.5</v>
       </c>
-      <c r="E9" s="57" t="str">
+      <c r="E9" s="109" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1260,18 +1567,18 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="11" t="str"/>
-      <c r="B10" s="11" t="str">
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="30" t="str"/>
+      <c r="B10" s="14" t="str">
         <v>Gạo tẻ</v>
       </c>
-      <c r="C10" s="12" t="str">
+      <c r="C10" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D10" s="69" t="n">
+      <c r="D10" s="93" t="n">
         <v>25</v>
       </c>
-      <c r="E10" s="57" t="str">
+      <c r="E10" s="109" t="str">
         <v>An Phú</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1335,18 +1642,18 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="29" customHeight="1">
-      <c r="A11" s="11" t="str"/>
-      <c r="B11" s="11" t="str">
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="30" t="str"/>
+      <c r="B11" s="14" t="str">
         <v>Thịt heo nạc</v>
       </c>
-      <c r="C11" s="12" t="str">
+      <c r="C11" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D11" s="55" t="n">
+      <c r="D11" s="79" t="n">
         <v>12.5</v>
       </c>
-      <c r="E11" s="57" t="str"/>
+      <c r="E11" s="109" t="str"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -1408,18 +1715,18 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="11" t="str"/>
-      <c r="B12" s="11" t="str">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="30" t="str"/>
+      <c r="B12" s="14" t="str">
         <v>Trứng gà</v>
       </c>
-      <c r="C12" s="12" t="str">
+      <c r="C12" s="15" t="str">
         <v>Quả</v>
       </c>
-      <c r="D12" s="69" t="n">
+      <c r="D12" s="93" t="n">
         <v>60</v>
       </c>
-      <c r="E12" s="57" t="str">
+      <c r="E12" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1483,18 +1790,18 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="11" t="str"/>
-      <c r="B13" s="11" t="str">
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="30" t="str"/>
+      <c r="B13" s="14" t="str">
         <v>Dầu ăn</v>
       </c>
-      <c r="C13" s="12" t="str">
+      <c r="C13" s="15" t="str">
         <v>Lít</v>
       </c>
-      <c r="D13" s="55" t="n">
+      <c r="D13" s="79" t="n">
         <v>2.5</v>
       </c>
-      <c r="E13" s="57" t="str">
+      <c r="E13" s="109" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1558,18 +1865,18 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="52" customHeight="1">
-      <c r="A14" s="11" t="str"/>
-      <c r="B14" s="11" t="str">
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="30" t="str"/>
+      <c r="B14" s="14" t="str">
         <v>Muối</v>
       </c>
-      <c r="C14" s="12" t="str">
+      <c r="C14" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D14" s="55" t="n">
+      <c r="D14" s="79" t="n">
         <v>0.5</v>
       </c>
-      <c r="E14" s="57" t="str">
+      <c r="E14" s="109" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1633,18 +1940,18 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="29" customHeight="1">
-      <c r="A15" s="11" t="str"/>
-      <c r="B15" s="11" t="str">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="30" t="str"/>
+      <c r="B15" s="14" t="str">
         <v>Nước mắm</v>
       </c>
-      <c r="C15" s="12" t="str">
+      <c r="C15" s="15" t="str">
         <v>Lít</v>
       </c>
-      <c r="D15" s="69" t="n">
+      <c r="D15" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="57" t="str"/>
+      <c r="E15" s="109" t="str"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -1706,18 +2013,18 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="70" customHeight="1">
-      <c r="A16" s="11" t="str"/>
-      <c r="B16" s="11" t="str">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="30" t="str"/>
+      <c r="B16" s="14" t="str">
         <v>Rau ngót</v>
       </c>
-      <c r="C16" s="12" t="str">
+      <c r="C16" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D16" s="55" t="n">
+      <c r="D16" s="79" t="n">
         <v>0.2</v>
       </c>
-      <c r="E16" s="57" t="str">
+      <c r="E16" s="109" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1781,18 +2088,18 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="11" t="str"/>
-      <c r="B17" s="11" t="str">
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="30" t="str"/>
+      <c r="B17" s="14" t="str">
         <v>Bí đỏ</v>
       </c>
-      <c r="C17" s="12" t="str">
+      <c r="C17" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D17" s="69" t="n">
+      <c r="D17" s="93" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="57" t="str">
+      <c r="E17" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1856,20 +2163,20 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="52" customHeight="1">
-      <c r="A18" s="19" t="str">
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="28" t="str">
         <v>Tân Định</v>
       </c>
-      <c r="B18" s="15" t="str">
+      <c r="B18" s="18" t="str">
         <v>Ớt hiểm đỏ</v>
       </c>
-      <c r="C18" s="16" t="str">
+      <c r="C18" s="19" t="str">
         <v>Kg</v>
       </c>
-      <c r="D18" s="63" t="n">
+      <c r="D18" s="87" t="n">
         <v>0.2</v>
       </c>
-      <c r="E18" s="65" t="str">
+      <c r="E18" s="105" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1933,18 +2240,18 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="11" t="str"/>
-      <c r="B19" s="11" t="str">
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="30" t="str"/>
+      <c r="B19" s="14" t="str">
         <v>Tỏi</v>
       </c>
-      <c r="C19" s="12" t="str">
+      <c r="C19" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D19" s="69" t="n">
+      <c r="D19" s="93" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="57" t="str">
+      <c r="E19" s="109" t="str">
         <v>An Phú</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -2008,18 +2315,18 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="70" customHeight="1">
-      <c r="A20" s="11" t="str"/>
-      <c r="B20" s="11" t="str">
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="30" t="str"/>
+      <c r="B20" s="14" t="str">
         <v>Cà rốt</v>
       </c>
-      <c r="C20" s="12" t="str">
+      <c r="C20" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D20" s="69" t="n">
+      <c r="D20" s="93" t="n">
         <v>3</v>
       </c>
-      <c r="E20" s="57" t="str">
+      <c r="E20" s="109" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -2083,18 +2390,18 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="11" t="str"/>
-      <c r="B21" s="11" t="str">
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="30" t="str"/>
+      <c r="B21" s="14" t="str">
         <v>Cải ngọt</v>
       </c>
-      <c r="C21" s="12" t="str">
+      <c r="C21" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D21" s="69" t="n">
+      <c r="D21" s="93" t="n">
         <v>7</v>
       </c>
-      <c r="E21" s="57" t="str">
+      <c r="E21" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -2158,18 +2465,18 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="11" t="str"/>
-      <c r="B22" s="11" t="str">
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="30" t="str"/>
+      <c r="B22" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
       </c>
-      <c r="C22" s="12" t="str">
+      <c r="C22" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D22" s="55" t="n">
+      <c r="D22" s="79" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E22" s="57" t="str">
+      <c r="E22" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -2233,20 +2540,20 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="52" customHeight="1">
-      <c r="A23" s="19" t="str">
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="28" t="str">
         <v>Tân Bình</v>
       </c>
-      <c r="B23" s="15" t="str">
+      <c r="B23" s="18" t="str">
         <v>Ớt hiểm đỏ</v>
       </c>
-      <c r="C23" s="16" t="str">
+      <c r="C23" s="19" t="str">
         <v>Kg</v>
       </c>
-      <c r="D23" s="63" t="n">
+      <c r="D23" s="87" t="n">
         <v>0.2</v>
       </c>
-      <c r="E23" s="65" t="str">
+      <c r="E23" s="105" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -2310,18 +2617,18 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="11" t="str"/>
-      <c r="B24" s="11" t="str">
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="30" t="str"/>
+      <c r="B24" s="14" t="str">
         <v>Tỏi</v>
       </c>
-      <c r="C24" s="12" t="str">
+      <c r="C24" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D24" s="69" t="n">
+      <c r="D24" s="93" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="57" t="str">
+      <c r="E24" s="109" t="str">
         <v>An Phú</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2385,18 +2692,18 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="70" customHeight="1">
-      <c r="A25" s="11" t="str"/>
-      <c r="B25" s="11" t="str">
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="30" t="str"/>
+      <c r="B25" s="14" t="str">
         <v>Cà rốt</v>
       </c>
-      <c r="C25" s="12" t="str">
+      <c r="C25" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D25" s="69" t="n">
+      <c r="D25" s="93" t="n">
         <v>3</v>
       </c>
-      <c r="E25" s="57" t="str">
+      <c r="E25" s="109" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -2460,18 +2767,18 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="11" t="str"/>
-      <c r="B26" s="11" t="str">
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="30" t="str"/>
+      <c r="B26" s="14" t="str">
         <v>Cải ngọt</v>
       </c>
-      <c r="C26" s="12" t="str">
+      <c r="C26" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D26" s="69" t="n">
+      <c r="D26" s="93" t="n">
         <v>7</v>
       </c>
-      <c r="E26" s="57" t="str">
+      <c r="E26" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -2535,18 +2842,18 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1">
-      <c r="A27" s="11" t="str"/>
-      <c r="B27" s="11" t="str">
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="30" t="str"/>
+      <c r="B27" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
       </c>
-      <c r="C27" s="12" t="str">
+      <c r="C27" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D27" s="55" t="n">
+      <c r="D27" s="79" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E27" s="57" t="str">
+      <c r="E27" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -2610,18 +2917,18 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="11" t="str"/>
-      <c r="B28" s="11" t="str">
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="30" t="str"/>
+      <c r="B28" s="14" t="str">
         <v>Hành lá</v>
       </c>
-      <c r="C28" s="12" t="str">
+      <c r="C28" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D28" s="55" t="n">
+      <c r="D28" s="79" t="n">
         <v>0.5</v>
       </c>
-      <c r="E28" s="57" t="str">
+      <c r="E28" s="109" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -2685,18 +2992,18 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="34" customHeight="1">
-      <c r="A29" s="11" t="str"/>
-      <c r="B29" s="11" t="str">
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="30" t="str"/>
+      <c r="B29" s="14" t="str">
         <v>Gạo tẻ</v>
       </c>
-      <c r="C29" s="12" t="str">
+      <c r="C29" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D29" s="69" t="n">
+      <c r="D29" s="93" t="n">
         <v>25</v>
       </c>
-      <c r="E29" s="57" t="str">
+      <c r="E29" s="109" t="str">
         <v>An Phú</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -2760,18 +3067,18 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="29" customHeight="1">
-      <c r="A30" s="11" t="str"/>
-      <c r="B30" s="11" t="str">
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="30" t="str"/>
+      <c r="B30" s="14" t="str">
         <v>Thịt heo nạc</v>
       </c>
-      <c r="C30" s="12" t="str">
+      <c r="C30" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D30" s="55" t="n">
+      <c r="D30" s="79" t="n">
         <v>12.5</v>
       </c>
-      <c r="E30" s="57" t="str"/>
+      <c r="E30" s="109" t="str"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -2833,18 +3140,18 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="34" customHeight="1">
-      <c r="A31" s="11" t="str"/>
-      <c r="B31" s="11" t="str">
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="30" t="str"/>
+      <c r="B31" s="14" t="str">
         <v>Trứng gà</v>
       </c>
-      <c r="C31" s="12" t="str">
+      <c r="C31" s="15" t="str">
         <v>Quả</v>
       </c>
-      <c r="D31" s="69" t="n">
+      <c r="D31" s="93" t="n">
         <v>60</v>
       </c>
-      <c r="E31" s="57" t="str">
+      <c r="E31" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2908,18 +3215,22 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="34" customHeight="1">
-      <c r="A32" s="11" t="str"/>
-      <c r="B32" s="11" t="str">
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="28" t="inlineStr">
+        <is>
+          <t>Tân Bình (tiếp)</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="str">
         <v>Dầu ăn</v>
       </c>
-      <c r="C32" s="12" t="str">
+      <c r="C32" s="15" t="str">
         <v>Lít</v>
       </c>
-      <c r="D32" s="55" t="n">
+      <c r="D32" s="79" t="n">
         <v>2.5</v>
       </c>
-      <c r="E32" s="57" t="str">
+      <c r="E32" s="109" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2983,18 +3294,18 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="52" customHeight="1">
-      <c r="A33" s="11" t="str"/>
-      <c r="B33" s="11" t="str">
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="30" t="str"/>
+      <c r="B33" s="14" t="str">
         <v>Muối</v>
       </c>
-      <c r="C33" s="12" t="str">
+      <c r="C33" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D33" s="55" t="n">
+      <c r="D33" s="79" t="n">
         <v>0.5</v>
       </c>
-      <c r="E33" s="57" t="str">
+      <c r="E33" s="109" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -3058,18 +3369,18 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="29" customHeight="1">
-      <c r="A34" s="11" t="str"/>
-      <c r="B34" s="11" t="str">
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="30" t="str"/>
+      <c r="B34" s="14" t="str">
         <v>Nước mắm</v>
       </c>
-      <c r="C34" s="12" t="str">
+      <c r="C34" s="15" t="str">
         <v>Lít</v>
       </c>
-      <c r="D34" s="69" t="n">
+      <c r="D34" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="E34" s="57" t="str"/>
+      <c r="E34" s="109" t="str"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -3131,22 +3442,18 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="70.0" customHeight="1">
-      <c r="A35" s="19" t="inlineStr">
-        <is>
-          <t>Tân Bình (tiếp)</t>
-        </is>
-      </c>
-      <c r="B35" s="11" t="str">
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" s="30" t="str"/>
+      <c r="B35" s="14" t="str">
         <v>Rau ngót</v>
       </c>
-      <c r="C35" s="12" t="str">
+      <c r="C35" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D35" s="55" t="n">
+      <c r="D35" s="79" t="n">
         <v>0.2</v>
       </c>
-      <c r="E35" s="57" t="str">
+      <c r="E35" s="109" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -3210,18 +3517,18 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="34" customHeight="1">
-      <c r="A36" s="11" t="str"/>
-      <c r="B36" s="11" t="str">
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" s="30" t="str"/>
+      <c r="B36" s="14" t="str">
         <v>Bí đỏ</v>
       </c>
-      <c r="C36" s="12" t="str">
+      <c r="C36" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D36" s="69" t="n">
+      <c r="D36" s="93" t="n">
         <v>1</v>
       </c>
-      <c r="E36" s="57" t="str">
+      <c r="E36" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -3285,18 +3592,18 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="34" customHeight="1">
-      <c r="A37" s="11" t="str"/>
-      <c r="B37" s="11" t="str">
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="30" t="str"/>
+      <c r="B37" s="14" t="str">
         <v>Khoai tây</v>
       </c>
-      <c r="C37" s="12" t="str">
+      <c r="C37" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D37" s="69" t="n">
+      <c r="D37" s="93" t="n">
         <v>3</v>
       </c>
-      <c r="E37" s="57" t="str">
+      <c r="E37" s="109" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -3360,18 +3667,18 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="29" customHeight="1">
-      <c r="A38" s="11" t="str"/>
-      <c r="B38" s="11" t="str">
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="30" t="str"/>
+      <c r="B38" s="14" t="str">
         <v>Cà chua</v>
       </c>
-      <c r="C38" s="12" t="str">
+      <c r="C38" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D38" s="69" t="n">
+      <c r="D38" s="93" t="n">
         <v>7</v>
       </c>
-      <c r="E38" s="57" t="str"/>
+      <c r="E38" s="109" t="str"/>
       <c r="F38" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -3433,18 +3740,18 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="34" customHeight="1">
-      <c r="A39" s="11" t="str"/>
-      <c r="B39" s="11" t="str">
+    <row r="39" ht="24" customHeight="1">
+      <c r="A39" s="30" t="str"/>
+      <c r="B39" s="14" t="str">
         <v>Cần ta</v>
       </c>
-      <c r="C39" s="12" t="str">
+      <c r="C39" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D39" s="69" t="n">
+      <c r="D39" s="93" t="n">
         <v>31</v>
       </c>
-      <c r="E39" s="57" t="str">
+      <c r="E39" s="109" t="str">
         <v>An Phú</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -3508,18 +3815,18 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="70" customHeight="1">
-      <c r="A40" s="11" t="str"/>
-      <c r="B40" s="11" t="str">
+    <row r="40" ht="24" customHeight="1">
+      <c r="A40" s="30" t="str"/>
+      <c r="B40" s="14" t="str">
         <v>Dưa leo</v>
       </c>
-      <c r="C40" s="12" t="str">
+      <c r="C40" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D40" s="55" t="n">
+      <c r="D40" s="79" t="n">
         <v>0.5</v>
       </c>
-      <c r="E40" s="57" t="str">
+      <c r="E40" s="109" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -3583,18 +3890,18 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="34" customHeight="1">
-      <c r="A41" s="11" t="str"/>
-      <c r="B41" s="11" t="str">
+    <row r="41" ht="24" customHeight="1">
+      <c r="A41" s="30" t="str"/>
+      <c r="B41" s="14" t="str">
         <v>Bắp cải</v>
       </c>
-      <c r="C41" s="12" t="str">
+      <c r="C41" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D41" s="69" t="n">
+      <c r="D41" s="93" t="n">
         <v>25</v>
       </c>
-      <c r="E41" s="57" t="str">
+      <c r="E41" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -3658,18 +3965,18 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="29" customHeight="1">
-      <c r="A42" s="11" t="str"/>
-      <c r="B42" s="11" t="str">
+    <row r="42" ht="24" customHeight="1">
+      <c r="A42" s="30" t="str"/>
+      <c r="B42" s="14" t="str">
         <v>Đậu cô ve</v>
       </c>
-      <c r="C42" s="12" t="str">
+      <c r="C42" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D42" s="55" t="n">
+      <c r="D42" s="79" t="n">
         <v>12.5</v>
       </c>
-      <c r="E42" s="57" t="str"/>
+      <c r="E42" s="109" t="str"/>
       <c r="F42" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -3731,18 +4038,18 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="52" customHeight="1">
-      <c r="A43" s="11" t="str"/>
-      <c r="B43" s="11" t="str">
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" s="30" t="str"/>
+      <c r="B43" s="14" t="str">
         <v>Su su</v>
       </c>
-      <c r="C43" s="12" t="str">
+      <c r="C43" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D43" s="69" t="n">
+      <c r="D43" s="93" t="n">
         <v>60</v>
       </c>
-      <c r="E43" s="57" t="str">
+      <c r="E43" s="109" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -3806,18 +4113,18 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="34" customHeight="1">
-      <c r="A44" s="11" t="str"/>
-      <c r="B44" s="11" t="str">
+    <row r="44" ht="24" customHeight="1">
+      <c r="A44" s="30" t="str"/>
+      <c r="B44" s="14" t="str">
         <v>Củ cải trắng</v>
       </c>
-      <c r="C44" s="12" t="str">
+      <c r="C44" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D44" s="55" t="n">
+      <c r="D44" s="79" t="n">
         <v>2.5</v>
       </c>
-      <c r="E44" s="57" t="str">
+      <c r="E44" s="109" t="str">
         <v>An Phú</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -3881,18 +4188,18 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="70" customHeight="1">
-      <c r="A45" s="11" t="str"/>
-      <c r="B45" s="11" t="str">
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="30" t="str"/>
+      <c r="B45" s="14" t="str">
         <v>Nấm rơm</v>
       </c>
-      <c r="C45" s="12" t="str">
+      <c r="C45" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D45" s="55" t="n">
+      <c r="D45" s="79" t="n">
         <v>0.5</v>
       </c>
-      <c r="E45" s="57" t="str">
+      <c r="E45" s="109" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -3956,18 +4263,18 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="29" customHeight="1">
-      <c r="A46" s="11" t="str"/>
-      <c r="B46" s="11" t="str">
+    <row r="46" ht="24" customHeight="1">
+      <c r="A46" s="30" t="str"/>
+      <c r="B46" s="14" t="str">
         <v>Sữa chua ăn</v>
       </c>
-      <c r="C46" s="12" t="str">
+      <c r="C46" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D46" s="55" t="n">
+      <c r="D46" s="79" t="n">
         <v>1.5</v>
       </c>
-      <c r="E46" s="57" t="str"/>
+      <c r="E46" s="109" t="str"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -4029,18 +4336,18 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="34" customHeight="1">
-      <c r="A47" s="11" t="str"/>
-      <c r="B47" s="11" t="str">
+    <row r="47" ht="24" customHeight="1">
+      <c r="A47" s="32" t="str"/>
+      <c r="B47" s="24" t="str">
         <v>Thịt gà phi lê</v>
       </c>
-      <c r="C47" s="12" t="str">
+      <c r="C47" s="25" t="str">
         <v>Kg</v>
       </c>
-      <c r="D47" s="55" t="n">
+      <c r="D47" s="99" t="n">
         <v>0.2</v>
       </c>
-      <c r="E47" s="57" t="str">
+      <c r="E47" s="113" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -4115,9 +4422,8 @@
   <headerFooter>
     <oddFooter>&amp;RTrang &amp;P / &amp;N</oddFooter>
   </headerFooter>
-  <rowBreaks count="2" manualBreakCount="2">
-    <brk id="17" min="0" max="16383" man="1"/>
-    <brk id="34" min="0" max="16383" man="1"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="31" min="0" max="16383" man="1"/>
   </rowBreaks>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -4132,15 +4438,15 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17.5" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="35" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="7.5" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="39" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="6.5" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="10.5" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="23" hidden="0" customWidth="1"/>
     <col min="6" max="17" width="1" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1" ht="29" customHeight="1">
       <c r="A1" s="4" t="str">
         <v>Thứ Ba (21/04/2026)</v>
       </c>
@@ -4161,7 +4467,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="9" customHeight="1">
+    <row r="2" ht="5" customHeight="1">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4180,20 +4486,20 @@
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
     </row>
-    <row r="3" ht="39" customHeight="1">
-      <c r="A3" s="25" t="str">
+    <row r="3" ht="29" customHeight="1">
+      <c r="A3" s="42" t="str">
         <v>TRƯỜNG</v>
       </c>
-      <c r="B3" s="26" t="str">
+      <c r="B3" s="43" t="str">
         <v>THÀNH PHẦN</v>
       </c>
-      <c r="C3" s="26" t="str">
+      <c r="C3" s="43" t="str">
         <v>ĐVT</v>
       </c>
-      <c r="D3" s="26" t="str">
+      <c r="D3" s="43" t="str">
         <v>SỐ LƯỢNG</v>
       </c>
-      <c r="E3" s="27" t="str">
+      <c r="E3" s="44" t="str">
         <v>GHI CHÚ</v>
       </c>
       <c r="F3" s="2" t="str">
@@ -4233,20 +4539,20 @@
         <v>__exported_note</v>
       </c>
     </row>
-    <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="19" t="str">
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="28" t="str">
         <v>Tân Định</v>
       </c>
-      <c r="B4" s="15" t="str">
+      <c r="B4" s="18" t="str">
         <v>Ớt hiểm đỏ</v>
       </c>
-      <c r="C4" s="16" t="str">
+      <c r="C4" s="19" t="str">
         <v>Kg</v>
       </c>
-      <c r="D4" s="63" t="n">
+      <c r="D4" s="87" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="65" t="str">
+      <c r="E4" s="105" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -4310,18 +4616,18 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="11" t="str"/>
-      <c r="B5" s="11" t="str">
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="30" t="str"/>
+      <c r="B5" s="14" t="str">
         <v>Tỏi</v>
       </c>
-      <c r="C5" s="12" t="str">
+      <c r="C5" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D5" s="69" t="n">
+      <c r="D5" s="93" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="57" t="str">
+      <c r="E5" s="109" t="str">
         <v>An Phú</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4385,18 +4691,18 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="11" t="str"/>
-      <c r="B6" s="11" t="str">
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="30" t="str"/>
+      <c r="B6" s="14" t="str">
         <v>Cà rốt</v>
       </c>
-      <c r="C6" s="12" t="str">
+      <c r="C6" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D6" s="69" t="n">
+      <c r="D6" s="93" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="57" t="str">
+      <c r="E6" s="109" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -4460,18 +4766,18 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="11" t="str"/>
-      <c r="B7" s="11" t="str">
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="30" t="str"/>
+      <c r="B7" s="14" t="str">
         <v>Cải ngọt</v>
       </c>
-      <c r="C7" s="12" t="str">
+      <c r="C7" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D7" s="69" t="n">
+      <c r="D7" s="93" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="57" t="str">
+      <c r="E7" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -4535,18 +4841,18 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="11" t="str"/>
-      <c r="B8" s="11" t="str">
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="30" t="str"/>
+      <c r="B8" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
       </c>
-      <c r="C8" s="12" t="str">
+      <c r="C8" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D8" s="55" t="n">
+      <c r="D8" s="79" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E8" s="57" t="str">
+      <c r="E8" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -4610,20 +4916,20 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="19" t="str">
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="28" t="str">
         <v>Tân Bình</v>
       </c>
-      <c r="B9" s="15" t="str">
+      <c r="B9" s="18" t="str">
         <v>Ớt hiểm đỏ</v>
       </c>
-      <c r="C9" s="16" t="str">
+      <c r="C9" s="19" t="str">
         <v>Kg</v>
       </c>
-      <c r="D9" s="63" t="n">
+      <c r="D9" s="87" t="n">
         <v>0.2</v>
       </c>
-      <c r="E9" s="65" t="str">
+      <c r="E9" s="105" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -4687,18 +4993,18 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="11" t="str"/>
-      <c r="B10" s="11" t="str">
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="30" t="str"/>
+      <c r="B10" s="14" t="str">
         <v>Tỏi</v>
       </c>
-      <c r="C10" s="12" t="str">
+      <c r="C10" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D10" s="69" t="n">
+      <c r="D10" s="93" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="57" t="str">
+      <c r="E10" s="109" t="str">
         <v>An Phú</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -4762,18 +5068,18 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="70" customHeight="1">
-      <c r="A11" s="11" t="str"/>
-      <c r="B11" s="11" t="str">
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="30" t="str"/>
+      <c r="B11" s="14" t="str">
         <v>Cà rốt</v>
       </c>
-      <c r="C11" s="12" t="str">
+      <c r="C11" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D11" s="69" t="n">
+      <c r="D11" s="93" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="57" t="str">
+      <c r="E11" s="109" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -4837,18 +5143,18 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="11" t="str"/>
-      <c r="B12" s="11" t="str">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="30" t="str"/>
+      <c r="B12" s="14" t="str">
         <v>Cải ngọt</v>
       </c>
-      <c r="C12" s="12" t="str">
+      <c r="C12" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D12" s="69" t="n">
+      <c r="D12" s="93" t="n">
         <v>7</v>
       </c>
-      <c r="E12" s="57" t="str">
+      <c r="E12" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -4912,18 +5218,18 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="11" t="str"/>
-      <c r="B13" s="11" t="str">
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="30" t="str"/>
+      <c r="B13" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
       </c>
-      <c r="C13" s="12" t="str">
+      <c r="C13" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D13" s="55" t="n">
+      <c r="D13" s="79" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E13" s="57" t="str">
+      <c r="E13" s="109" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -4987,18 +5293,18 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="11" t="str"/>
-      <c r="B14" s="11" t="str">
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="30" t="str"/>
+      <c r="B14" s="14" t="str">
         <v>Hành lá</v>
       </c>
-      <c r="C14" s="12" t="str">
+      <c r="C14" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D14" s="55" t="n">
+      <c r="D14" s="79" t="n">
         <v>0.5</v>
       </c>
-      <c r="E14" s="57" t="str">
+      <c r="E14" s="109" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -5062,18 +5368,18 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="11" t="str"/>
-      <c r="B15" s="11" t="str">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="32" t="str"/>
+      <c r="B15" s="24" t="str">
         <v>Gạo tẻ</v>
       </c>
-      <c r="C15" s="12" t="str">
+      <c r="C15" s="25" t="str">
         <v>Kg</v>
       </c>
-      <c r="D15" s="69" t="n">
+      <c r="D15" s="137" t="n">
         <v>25</v>
       </c>
-      <c r="E15" s="57" t="str">
+      <c r="E15" s="113" t="str">
         <v>An Phú</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -5164,120 +5470,120 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="46" t="inlineStr">
         <is>
           <t>contract_name</t>
         </is>
       </c>
-      <c r="B1" s="28" t="inlineStr">
+      <c r="B1" s="46" t="inlineStr">
         <is>
           <t>ATLAS_SHOPPING_LIST</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="46" t="inlineStr">
         <is>
           <t>contract_version</t>
         </is>
       </c>
-      <c r="B2" s="28" t="inlineStr">
+      <c r="B2" s="46" t="inlineStr">
         <is>
           <t>ATLAS_SHOPPING_LIST_V1</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="46" t="inlineStr">
         <is>
           <t>workbook_marker</t>
         </is>
       </c>
-      <c r="B3" s="28" t="inlineStr">
+      <c r="B3" s="46" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>exported_at</t>
         </is>
       </c>
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="46" t="inlineStr">
         <is>
           <t>2026-04-19T10:00:00.000Z</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>service_period_start</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="46" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>service_period_end</t>
         </is>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="46" t="inlineStr">
         <is>
           <t>2026-04-21</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="46" t="inlineStr">
         <is>
           <t>confirmed_need_batch_id</t>
         </is>
       </c>
-      <c r="B7" s="28" t="inlineStr">
+      <c r="B7" s="46" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000000001</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="46" t="inlineStr">
         <is>
           <t>batch_version</t>
         </is>
       </c>
-      <c r="B8" s="28" t="inlineStr">
+      <c r="B8" s="46" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="46" t="inlineStr">
         <is>
           <t>need_generation_run_id</t>
         </is>
       </c>
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B9" s="46" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000000002</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="46" t="inlineStr">
         <is>
           <t>release_snapshot_id</t>
         </is>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="46" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000000003</t>
         </is>

</xml_diff>

<commit_message>
docs(atlas): simplify Shopping List XLSX v1 daily contract
</commit_message>
<xml_diff>
--- a/docs/xlsx/examples/atlas-shopping-list-v1-example.xlsx
+++ b/docs/xlsx/examples/atlas-shopping-list-v1-example.xlsx
@@ -5,13 +5,16 @@
   <sheets>
     <sheet name="2026-04-20" sheetId="1" r:id="rId4"/>
     <sheet name="2026-04-21" sheetId="2" r:id="rId5"/>
-    <sheet name="_ATLAS_META" sheetId="3" r:id="rId6" state="veryHidden"/>
+    <sheet name="2026-04-22" sheetId="3" r:id="rId6"/>
+    <sheet name="_ATLAS_META" sheetId="4" r:id="rId7" state="veryHidden"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'2026-04-20'!$A$1:$E$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'2026-04-20'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'2026-04-21'!$A$1:$E$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'2026-04-21'!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'2026-04-22'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'2026-04-22'!$1:$3</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -251,7 +254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="144">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -386,6 +389,9 @@
     <xf numFmtId="201" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
     </xf>
+    <xf numFmtId="201" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -748,6 +754,14 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="201" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
@@ -765,9 +779,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AtlasNeed_20260420" displayName="AtlasNeed_20260420" ref="A3:Q47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A3:Q47"/>
-  <tableColumns count="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AtlasNeed_20260420" displayName="AtlasNeed_20260420" ref="A3:O47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A3:O47"/>
+  <tableColumns count="15">
     <tableColumn id="1" name="TRƯỜNG"/>
     <tableColumn id="2" name="THÀNH PHẦN"/>
     <tableColumn id="3" name="ĐVT"/>
@@ -783,17 +797,15 @@
     <tableColumn id="13" name="__ingredient_id"/>
     <tableColumn id="14" name="__unit_id"/>
     <tableColumn id="15" name="__exported_quantity"/>
-    <tableColumn id="16" name="__exported_reason_code"/>
-    <tableColumn id="17" name="__exported_note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AtlasNeed_20260421" displayName="AtlasNeed_20260421" ref="A3:Q15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A3:Q15"/>
-  <tableColumns count="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AtlasNeed_20260421" displayName="AtlasNeed_20260421" ref="A3:O15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A3:O15"/>
+  <tableColumns count="15">
     <tableColumn id="1" name="TRƯỜNG"/>
     <tableColumn id="2" name="THÀNH PHẦN"/>
     <tableColumn id="3" name="ĐVT"/>
@@ -809,8 +821,30 @@
     <tableColumn id="13" name="__ingredient_id"/>
     <tableColumn id="14" name="__unit_id"/>
     <tableColumn id="15" name="__exported_quantity"/>
-    <tableColumn id="16" name="__exported_reason_code"/>
-    <tableColumn id="17" name="__exported_note"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AtlasNeed_20260422" displayName="AtlasNeed_20260422" ref="A3:O6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A3:O6"/>
+  <tableColumns count="15">
+    <tableColumn id="1" name="TRƯỜNG"/>
+    <tableColumn id="2" name="THÀNH PHẦN"/>
+    <tableColumn id="3" name="ĐVT"/>
+    <tableColumn id="4" name="SỐ LƯỢNG"/>
+    <tableColumn id="5" name="GHI CHÚ"/>
+    <tableColumn id="6" name="__workbook_marker"/>
+    <tableColumn id="7" name="__line_id"/>
+    <tableColumn id="8" name="__revision_id"/>
+    <tableColumn id="9" name="__decision_id"/>
+    <tableColumn id="10" name="__service_date"/>
+    <tableColumn id="11" name="__school_id"/>
+    <tableColumn id="12" name="__location_id"/>
+    <tableColumn id="13" name="__ingredient_id"/>
+    <tableColumn id="14" name="__unit_id"/>
+    <tableColumn id="15" name="__exported_quantity"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -1019,7 +1053,7 @@
     <col min="3" max="3" width="6.5" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="10.5" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="23" hidden="0" customWidth="1"/>
-    <col min="6" max="17" width="1" customWidth="1" hidden="1"/>
+    <col min="6" max="15" width="1" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="29" customHeight="1">
@@ -1040,8 +1074,6 @@
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
     </row>
     <row r="2" ht="5" customHeight="1">
       <c r="A2" s="2"/>
@@ -1059,8 +1091,6 @@
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
     </row>
     <row r="3" ht="29" customHeight="1">
       <c r="A3" s="42" t="str">
@@ -1108,12 +1138,6 @@
       <c r="O3" s="2" t="str">
         <v>__exported_quantity</v>
       </c>
-      <c r="P3" s="2" t="str">
-        <v>__exported_reason_code</v>
-      </c>
-      <c r="Q3" s="2" t="str">
-        <v>__exported_note</v>
-      </c>
     </row>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="28" t="str">
@@ -1125,10 +1149,10 @@
       <c r="C4" s="19" t="str">
         <v>Kg</v>
       </c>
-      <c r="D4" s="87" t="n">
+      <c r="D4" s="88" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="105" t="str">
+      <c r="E4" s="106" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1179,16 +1203,6 @@
       <c r="O4" s="2" t="inlineStr">
         <is>
           <t>0.2</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q4" s="2" t="inlineStr">
-        <is>
-          <t>Công ty Hoàng Dung Dairy</t>
         </is>
       </c>
     </row>
@@ -1200,10 +1214,10 @@
       <c r="C5" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D5" s="93" t="n">
+      <c r="D5" s="94" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="109" t="str">
+      <c r="E5" s="110" t="str">
         <v>An Phú</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1254,16 +1268,6 @@
       <c r="O5" s="2" t="inlineStr">
         <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="inlineStr">
-        <is>
-          <t>OPERATIONAL_QUANTITY_ADJUSTMENT</t>
-        </is>
-      </c>
-      <c r="Q5" s="2" t="inlineStr">
-        <is>
-          <t>An Phú</t>
         </is>
       </c>
     </row>
@@ -1275,10 +1279,10 @@
       <c r="C6" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D6" s="93" t="n">
+      <c r="D6" s="94" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="109" t="str">
+      <c r="E6" s="110" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1329,16 +1333,6 @@
       <c r="O6" s="2" t="inlineStr">
         <is>
           <t>3</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q6" s="2" t="inlineStr">
-        <is>
-          <t>Nông sản Bình Minh - giao bếp trường mỗi sáng</t>
         </is>
       </c>
     </row>
@@ -1350,10 +1344,10 @@
       <c r="C7" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D7" s="93" t="n">
+      <c r="D7" s="94" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="109" t="str">
+      <c r="E7" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1404,16 +1398,6 @@
       <c r="O7" s="2" t="inlineStr">
         <is>
           <t>7</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q7" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -1425,10 +1409,10 @@
       <c r="C8" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D8" s="79" t="n">
+      <c r="D8" s="80" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E8" s="109" t="str">
+      <c r="E8" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1479,16 +1463,6 @@
       <c r="O8" s="2" t="inlineStr">
         <is>
           <t>1.234567</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q8" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -1500,10 +1474,10 @@
       <c r="C9" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D9" s="79" t="n">
+      <c r="D9" s="80" t="n">
         <v>0.5</v>
       </c>
-      <c r="E9" s="109" t="str">
+      <c r="E9" s="110" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1554,16 +1528,6 @@
       <c r="O9" s="2" t="inlineStr">
         <is>
           <t>0.5</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q9" s="2" t="inlineStr">
-        <is>
-          <t>Chợ A</t>
         </is>
       </c>
     </row>
@@ -1575,10 +1539,10 @@
       <c r="C10" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D10" s="93" t="n">
+      <c r="D10" s="94" t="n">
         <v>25</v>
       </c>
-      <c r="E10" s="109" t="str">
+      <c r="E10" s="110" t="str">
         <v>An Phú</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1629,16 +1593,6 @@
       <c r="O10" s="2" t="inlineStr">
         <is>
           <t>25</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q10" s="2" t="inlineStr">
-        <is>
-          <t>An Phú</t>
         </is>
       </c>
     </row>
@@ -1650,10 +1604,10 @@
       <c r="C11" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D11" s="79" t="n">
+      <c r="D11" s="80" t="n">
         <v>12.5</v>
       </c>
-      <c r="E11" s="109" t="str"/>
+      <c r="E11" s="110" t="str"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -1702,16 +1656,6 @@
       <c r="O11" s="2" t="inlineStr">
         <is>
           <t>12.5</t>
-        </is>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q11" s="2" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
     </row>
@@ -1723,10 +1667,10 @@
       <c r="C12" s="15" t="str">
         <v>Quả</v>
       </c>
-      <c r="D12" s="93" t="n">
+      <c r="D12" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="E12" s="109" t="str">
+      <c r="E12" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1777,16 +1721,6 @@
       <c r="O12" s="2" t="inlineStr">
         <is>
           <t>60</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q12" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -1798,10 +1732,10 @@
       <c r="C13" s="15" t="str">
         <v>Lít</v>
       </c>
-      <c r="D13" s="79" t="n">
+      <c r="D13" s="80" t="n">
         <v>2.5</v>
       </c>
-      <c r="E13" s="109" t="str">
+      <c r="E13" s="110" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1852,16 +1786,6 @@
       <c r="O13" s="2" t="inlineStr">
         <is>
           <t>2.5</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q13" s="2" t="inlineStr">
-        <is>
-          <t>Chợ A</t>
         </is>
       </c>
     </row>
@@ -1873,10 +1797,10 @@
       <c r="C14" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D14" s="79" t="n">
+      <c r="D14" s="80" t="n">
         <v>0.5</v>
       </c>
-      <c r="E14" s="109" t="str">
+      <c r="E14" s="110" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1927,16 +1851,6 @@
       <c r="O14" s="2" t="inlineStr">
         <is>
           <t>0.5</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q14" s="2" t="inlineStr">
-        <is>
-          <t>Công ty Hoàng Dung Dairy</t>
         </is>
       </c>
     </row>
@@ -1948,10 +1862,10 @@
       <c r="C15" s="15" t="str">
         <v>Lít</v>
       </c>
-      <c r="D15" s="93" t="n">
+      <c r="D15" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="109" t="str"/>
+      <c r="E15" s="110" t="str"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -2000,16 +1914,6 @@
       <c r="O15" s="2" t="inlineStr">
         <is>
           <t>0</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q15" s="2" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
     </row>
@@ -2021,10 +1925,10 @@
       <c r="C16" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D16" s="79" t="n">
+      <c r="D16" s="80" t="n">
         <v>0.2</v>
       </c>
-      <c r="E16" s="109" t="str">
+      <c r="E16" s="110" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -2075,16 +1979,6 @@
       <c r="O16" s="2" t="inlineStr">
         <is>
           <t>0.2</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q16" s="2" t="inlineStr">
-        <is>
-          <t>Nông sản Bình Minh - giao bếp trường mỗi sáng</t>
         </is>
       </c>
     </row>
@@ -2096,10 +1990,10 @@
       <c r="C17" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D17" s="93" t="n">
+      <c r="D17" s="94" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="109" t="str">
+      <c r="E17" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -2150,16 +2044,6 @@
       <c r="O17" s="2" t="inlineStr">
         <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q17" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -2173,10 +2057,10 @@
       <c r="C18" s="19" t="str">
         <v>Kg</v>
       </c>
-      <c r="D18" s="87" t="n">
+      <c r="D18" s="88" t="n">
         <v>0.2</v>
       </c>
-      <c r="E18" s="105" t="str">
+      <c r="E18" s="106" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -2227,16 +2111,6 @@
       <c r="O18" s="2" t="inlineStr">
         <is>
           <t>0.2</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q18" s="2" t="inlineStr">
-        <is>
-          <t>Công ty Hoàng Dung Dairy</t>
         </is>
       </c>
     </row>
@@ -2248,10 +2122,10 @@
       <c r="C19" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D19" s="93" t="n">
+      <c r="D19" s="94" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="109" t="str">
+      <c r="E19" s="110" t="str">
         <v>An Phú</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -2302,16 +2176,6 @@
       <c r="O19" s="2" t="inlineStr">
         <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>OPERATIONAL_QUANTITY_ADJUSTMENT</t>
-        </is>
-      </c>
-      <c r="Q19" s="2" t="inlineStr">
-        <is>
-          <t>An Phú</t>
         </is>
       </c>
     </row>
@@ -2323,10 +2187,10 @@
       <c r="C20" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D20" s="93" t="n">
+      <c r="D20" s="94" t="n">
         <v>3</v>
       </c>
-      <c r="E20" s="109" t="str">
+      <c r="E20" s="110" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -2377,16 +2241,6 @@
       <c r="O20" s="2" t="inlineStr">
         <is>
           <t>3</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q20" s="2" t="inlineStr">
-        <is>
-          <t>Nông sản Bình Minh - giao bếp trường mỗi sáng</t>
         </is>
       </c>
     </row>
@@ -2398,10 +2252,10 @@
       <c r="C21" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D21" s="93" t="n">
+      <c r="D21" s="94" t="n">
         <v>7</v>
       </c>
-      <c r="E21" s="109" t="str">
+      <c r="E21" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -2452,16 +2306,6 @@
       <c r="O21" s="2" t="inlineStr">
         <is>
           <t>7</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q21" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -2473,10 +2317,10 @@
       <c r="C22" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D22" s="79" t="n">
+      <c r="D22" s="80" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E22" s="109" t="str">
+      <c r="E22" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -2527,16 +2371,6 @@
       <c r="O22" s="2" t="inlineStr">
         <is>
           <t>1.234567</t>
-        </is>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q22" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -2550,10 +2384,10 @@
       <c r="C23" s="19" t="str">
         <v>Kg</v>
       </c>
-      <c r="D23" s="87" t="n">
+      <c r="D23" s="88" t="n">
         <v>0.2</v>
       </c>
-      <c r="E23" s="105" t="str">
+      <c r="E23" s="106" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -2604,16 +2438,6 @@
       <c r="O23" s="2" t="inlineStr">
         <is>
           <t>0.2</t>
-        </is>
-      </c>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q23" s="2" t="inlineStr">
-        <is>
-          <t>Công ty Hoàng Dung Dairy</t>
         </is>
       </c>
     </row>
@@ -2625,10 +2449,10 @@
       <c r="C24" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D24" s="93" t="n">
+      <c r="D24" s="94" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="109" t="str">
+      <c r="E24" s="110" t="str">
         <v>An Phú</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2679,16 +2503,6 @@
       <c r="O24" s="2" t="inlineStr">
         <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="P24" s="2" t="inlineStr">
-        <is>
-          <t>OPERATIONAL_QUANTITY_ADJUSTMENT</t>
-        </is>
-      </c>
-      <c r="Q24" s="2" t="inlineStr">
-        <is>
-          <t>An Phú</t>
         </is>
       </c>
     </row>
@@ -2700,10 +2514,10 @@
       <c r="C25" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D25" s="93" t="n">
+      <c r="D25" s="94" t="n">
         <v>3</v>
       </c>
-      <c r="E25" s="109" t="str">
+      <c r="E25" s="110" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -2754,16 +2568,6 @@
       <c r="O25" s="2" t="inlineStr">
         <is>
           <t>3</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q25" s="2" t="inlineStr">
-        <is>
-          <t>Nông sản Bình Minh - giao bếp trường mỗi sáng</t>
         </is>
       </c>
     </row>
@@ -2775,10 +2579,10 @@
       <c r="C26" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D26" s="93" t="n">
+      <c r="D26" s="94" t="n">
         <v>7</v>
       </c>
-      <c r="E26" s="109" t="str">
+      <c r="E26" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -2829,16 +2633,6 @@
       <c r="O26" s="2" t="inlineStr">
         <is>
           <t>7</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q26" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -2850,10 +2644,10 @@
       <c r="C27" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D27" s="79" t="n">
+      <c r="D27" s="80" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E27" s="109" t="str">
+      <c r="E27" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -2904,16 +2698,6 @@
       <c r="O27" s="2" t="inlineStr">
         <is>
           <t>1.234567</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q27" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -2925,10 +2709,10 @@
       <c r="C28" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D28" s="79" t="n">
+      <c r="D28" s="80" t="n">
         <v>0.5</v>
       </c>
-      <c r="E28" s="109" t="str">
+      <c r="E28" s="110" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -2979,16 +2763,6 @@
       <c r="O28" s="2" t="inlineStr">
         <is>
           <t>0.5</t>
-        </is>
-      </c>
-      <c r="P28" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q28" s="2" t="inlineStr">
-        <is>
-          <t>Chợ A</t>
         </is>
       </c>
     </row>
@@ -3000,10 +2774,10 @@
       <c r="C29" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D29" s="93" t="n">
+      <c r="D29" s="94" t="n">
         <v>25</v>
       </c>
-      <c r="E29" s="109" t="str">
+      <c r="E29" s="110" t="str">
         <v>An Phú</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -3054,16 +2828,6 @@
       <c r="O29" s="2" t="inlineStr">
         <is>
           <t>25</t>
-        </is>
-      </c>
-      <c r="P29" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q29" s="2" t="inlineStr">
-        <is>
-          <t>An Phú</t>
         </is>
       </c>
     </row>
@@ -3075,10 +2839,10 @@
       <c r="C30" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D30" s="79" t="n">
+      <c r="D30" s="80" t="n">
         <v>12.5</v>
       </c>
-      <c r="E30" s="109" t="str"/>
+      <c r="E30" s="110" t="str"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -3127,16 +2891,6 @@
       <c r="O30" s="2" t="inlineStr">
         <is>
           <t>12.5</t>
-        </is>
-      </c>
-      <c r="P30" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q30" s="2" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
     </row>
@@ -3148,10 +2902,10 @@
       <c r="C31" s="15" t="str">
         <v>Quả</v>
       </c>
-      <c r="D31" s="93" t="n">
+      <c r="D31" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="E31" s="109" t="str">
+      <c r="E31" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -3202,16 +2956,6 @@
       <c r="O31" s="2" t="inlineStr">
         <is>
           <t>60</t>
-        </is>
-      </c>
-      <c r="P31" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q31" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -3227,10 +2971,10 @@
       <c r="C32" s="15" t="str">
         <v>Lít</v>
       </c>
-      <c r="D32" s="79" t="n">
+      <c r="D32" s="80" t="n">
         <v>2.5</v>
       </c>
-      <c r="E32" s="109" t="str">
+      <c r="E32" s="110" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -3281,16 +3025,6 @@
       <c r="O32" s="2" t="inlineStr">
         <is>
           <t>2.5</t>
-        </is>
-      </c>
-      <c r="P32" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q32" s="2" t="inlineStr">
-        <is>
-          <t>Chợ A</t>
         </is>
       </c>
     </row>
@@ -3302,10 +3036,10 @@
       <c r="C33" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D33" s="79" t="n">
+      <c r="D33" s="80" t="n">
         <v>0.5</v>
       </c>
-      <c r="E33" s="109" t="str">
+      <c r="E33" s="110" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -3356,16 +3090,6 @@
       <c r="O33" s="2" t="inlineStr">
         <is>
           <t>0.5</t>
-        </is>
-      </c>
-      <c r="P33" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q33" s="2" t="inlineStr">
-        <is>
-          <t>Công ty Hoàng Dung Dairy</t>
         </is>
       </c>
     </row>
@@ -3377,10 +3101,10 @@
       <c r="C34" s="15" t="str">
         <v>Lít</v>
       </c>
-      <c r="D34" s="93" t="n">
+      <c r="D34" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="E34" s="109" t="str"/>
+      <c r="E34" s="110" t="str"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -3429,16 +3153,6 @@
       <c r="O34" s="2" t="inlineStr">
         <is>
           <t>0</t>
-        </is>
-      </c>
-      <c r="P34" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q34" s="2" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
     </row>
@@ -3450,10 +3164,10 @@
       <c r="C35" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D35" s="79" t="n">
+      <c r="D35" s="80" t="n">
         <v>0.2</v>
       </c>
-      <c r="E35" s="109" t="str">
+      <c r="E35" s="110" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -3504,16 +3218,6 @@
       <c r="O35" s="2" t="inlineStr">
         <is>
           <t>0.2</t>
-        </is>
-      </c>
-      <c r="P35" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q35" s="2" t="inlineStr">
-        <is>
-          <t>Nông sản Bình Minh - giao bếp trường mỗi sáng</t>
         </is>
       </c>
     </row>
@@ -3525,10 +3229,10 @@
       <c r="C36" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D36" s="93" t="n">
+      <c r="D36" s="94" t="n">
         <v>1</v>
       </c>
-      <c r="E36" s="109" t="str">
+      <c r="E36" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -3579,16 +3283,6 @@
       <c r="O36" s="2" t="inlineStr">
         <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="P36" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q36" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -3600,10 +3294,10 @@
       <c r="C37" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D37" s="93" t="n">
+      <c r="D37" s="94" t="n">
         <v>3</v>
       </c>
-      <c r="E37" s="109" t="str">
+      <c r="E37" s="110" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -3654,16 +3348,6 @@
       <c r="O37" s="2" t="inlineStr">
         <is>
           <t>3</t>
-        </is>
-      </c>
-      <c r="P37" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q37" s="2" t="inlineStr">
-        <is>
-          <t>Chợ A</t>
         </is>
       </c>
     </row>
@@ -3675,10 +3359,10 @@
       <c r="C38" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D38" s="93" t="n">
+      <c r="D38" s="94" t="n">
         <v>7</v>
       </c>
-      <c r="E38" s="109" t="str"/>
+      <c r="E38" s="110" t="str"/>
       <c r="F38" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -3727,16 +3411,6 @@
       <c r="O38" s="2" t="inlineStr">
         <is>
           <t>7</t>
-        </is>
-      </c>
-      <c r="P38" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q38" s="2" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
     </row>
@@ -3748,10 +3422,10 @@
       <c r="C39" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D39" s="93" t="n">
+      <c r="D39" s="94" t="n">
         <v>31</v>
       </c>
-      <c r="E39" s="109" t="str">
+      <c r="E39" s="110" t="str">
         <v>An Phú</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -3802,16 +3476,6 @@
       <c r="O39" s="2" t="inlineStr">
         <is>
           <t>31</t>
-        </is>
-      </c>
-      <c r="P39" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q39" s="2" t="inlineStr">
-        <is>
-          <t>An Phú</t>
         </is>
       </c>
     </row>
@@ -3823,10 +3487,10 @@
       <c r="C40" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D40" s="79" t="n">
+      <c r="D40" s="80" t="n">
         <v>0.5</v>
       </c>
-      <c r="E40" s="109" t="str">
+      <c r="E40" s="110" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -3877,16 +3541,6 @@
       <c r="O40" s="2" t="inlineStr">
         <is>
           <t>0.5</t>
-        </is>
-      </c>
-      <c r="P40" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q40" s="2" t="inlineStr">
-        <is>
-          <t>Nông sản Bình Minh - giao bếp trường mỗi sáng</t>
         </is>
       </c>
     </row>
@@ -3898,10 +3552,10 @@
       <c r="C41" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D41" s="93" t="n">
+      <c r="D41" s="94" t="n">
         <v>25</v>
       </c>
-      <c r="E41" s="109" t="str">
+      <c r="E41" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -3952,16 +3606,6 @@
       <c r="O41" s="2" t="inlineStr">
         <is>
           <t>25</t>
-        </is>
-      </c>
-      <c r="P41" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q41" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -3973,10 +3617,10 @@
       <c r="C42" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D42" s="79" t="n">
+      <c r="D42" s="80" t="n">
         <v>12.5</v>
       </c>
-      <c r="E42" s="109" t="str"/>
+      <c r="E42" s="110" t="str"/>
       <c r="F42" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -4025,16 +3669,6 @@
       <c r="O42" s="2" t="inlineStr">
         <is>
           <t>12.5</t>
-        </is>
-      </c>
-      <c r="P42" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q42" s="2" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
     </row>
@@ -4046,10 +3680,10 @@
       <c r="C43" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D43" s="93" t="n">
+      <c r="D43" s="94" t="n">
         <v>60</v>
       </c>
-      <c r="E43" s="109" t="str">
+      <c r="E43" s="110" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -4100,16 +3734,6 @@
       <c r="O43" s="2" t="inlineStr">
         <is>
           <t>60</t>
-        </is>
-      </c>
-      <c r="P43" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q43" s="2" t="inlineStr">
-        <is>
-          <t>Công ty Hoàng Dung Dairy</t>
         </is>
       </c>
     </row>
@@ -4121,10 +3745,10 @@
       <c r="C44" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D44" s="79" t="n">
+      <c r="D44" s="80" t="n">
         <v>2.5</v>
       </c>
-      <c r="E44" s="109" t="str">
+      <c r="E44" s="110" t="str">
         <v>An Phú</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -4175,16 +3799,6 @@
       <c r="O44" s="2" t="inlineStr">
         <is>
           <t>2.5</t>
-        </is>
-      </c>
-      <c r="P44" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q44" s="2" t="inlineStr">
-        <is>
-          <t>An Phú</t>
         </is>
       </c>
     </row>
@@ -4196,10 +3810,10 @@
       <c r="C45" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D45" s="79" t="n">
+      <c r="D45" s="80" t="n">
         <v>0.5</v>
       </c>
-      <c r="E45" s="109" t="str">
+      <c r="E45" s="110" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -4250,16 +3864,6 @@
       <c r="O45" s="2" t="inlineStr">
         <is>
           <t>0.5</t>
-        </is>
-      </c>
-      <c r="P45" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q45" s="2" t="inlineStr">
-        <is>
-          <t>Nông sản Bình Minh - giao bếp trường mỗi sáng</t>
         </is>
       </c>
     </row>
@@ -4271,10 +3875,10 @@
       <c r="C46" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D46" s="79" t="n">
+      <c r="D46" s="80" t="n">
         <v>1.5</v>
       </c>
-      <c r="E46" s="109" t="str"/>
+      <c r="E46" s="110" t="str"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -4323,16 +3927,6 @@
       <c r="O46" s="2" t="inlineStr">
         <is>
           <t>1.5</t>
-        </is>
-      </c>
-      <c r="P46" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q46" s="2" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
     </row>
@@ -4344,10 +3938,10 @@
       <c r="C47" s="25" t="str">
         <v>Kg</v>
       </c>
-      <c r="D47" s="99" t="n">
+      <c r="D47" s="100" t="n">
         <v>0.2</v>
       </c>
-      <c r="E47" s="113" t="str">
+      <c r="E47" s="114" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -4398,16 +3992,6 @@
       <c r="O47" s="2" t="inlineStr">
         <is>
           <t>0.2</t>
-        </is>
-      </c>
-      <c r="P47" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q47" s="2" t="inlineStr">
-        <is>
-          <t>Chợ A</t>
         </is>
       </c>
     </row>
@@ -4443,7 +4027,7 @@
     <col min="3" max="3" width="6.5" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="10.5" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="23" hidden="0" customWidth="1"/>
-    <col min="6" max="17" width="1" customWidth="1" hidden="1"/>
+    <col min="6" max="15" width="1" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="29" customHeight="1">
@@ -4464,8 +4048,6 @@
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
     </row>
     <row r="2" ht="5" customHeight="1">
       <c r="A2" s="2"/>
@@ -4483,8 +4065,6 @@
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
     </row>
     <row r="3" ht="29" customHeight="1">
       <c r="A3" s="42" t="str">
@@ -4532,12 +4112,6 @@
       <c r="O3" s="2" t="str">
         <v>__exported_quantity</v>
       </c>
-      <c r="P3" s="2" t="str">
-        <v>__exported_reason_code</v>
-      </c>
-      <c r="Q3" s="2" t="str">
-        <v>__exported_note</v>
-      </c>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="28" t="str">
@@ -4549,10 +4123,10 @@
       <c r="C4" s="19" t="str">
         <v>Kg</v>
       </c>
-      <c r="D4" s="87" t="n">
+      <c r="D4" s="88" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="105" t="str">
+      <c r="E4" s="106" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -4603,16 +4177,6 @@
       <c r="O4" s="2" t="inlineStr">
         <is>
           <t>0.2</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q4" s="2" t="inlineStr">
-        <is>
-          <t>Công ty Hoàng Dung Dairy</t>
         </is>
       </c>
     </row>
@@ -4624,10 +4188,10 @@
       <c r="C5" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D5" s="93" t="n">
+      <c r="D5" s="94" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="109" t="str">
+      <c r="E5" s="110" t="str">
         <v>An Phú</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4678,16 +4242,6 @@
       <c r="O5" s="2" t="inlineStr">
         <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="inlineStr">
-        <is>
-          <t>OPERATIONAL_QUANTITY_ADJUSTMENT</t>
-        </is>
-      </c>
-      <c r="Q5" s="2" t="inlineStr">
-        <is>
-          <t>An Phú</t>
         </is>
       </c>
     </row>
@@ -4699,10 +4253,10 @@
       <c r="C6" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D6" s="93" t="n">
+      <c r="D6" s="94" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="109" t="str">
+      <c r="E6" s="110" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -4753,16 +4307,6 @@
       <c r="O6" s="2" t="inlineStr">
         <is>
           <t>3</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q6" s="2" t="inlineStr">
-        <is>
-          <t>Nông sản Bình Minh - giao bếp trường mỗi sáng</t>
         </is>
       </c>
     </row>
@@ -4774,10 +4318,10 @@
       <c r="C7" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D7" s="93" t="n">
+      <c r="D7" s="94" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="109" t="str">
+      <c r="E7" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -4828,16 +4372,6 @@
       <c r="O7" s="2" t="inlineStr">
         <is>
           <t>7</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q7" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -4849,10 +4383,10 @@
       <c r="C8" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D8" s="79" t="n">
+      <c r="D8" s="80" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E8" s="109" t="str">
+      <c r="E8" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -4903,16 +4437,6 @@
       <c r="O8" s="2" t="inlineStr">
         <is>
           <t>1.234567</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q8" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -4926,10 +4450,10 @@
       <c r="C9" s="19" t="str">
         <v>Kg</v>
       </c>
-      <c r="D9" s="87" t="n">
+      <c r="D9" s="88" t="n">
         <v>0.2</v>
       </c>
-      <c r="E9" s="105" t="str">
+      <c r="E9" s="106" t="str">
         <v>Công ty Hoàng Dung Dairy</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -4980,16 +4504,6 @@
       <c r="O9" s="2" t="inlineStr">
         <is>
           <t>0.2</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q9" s="2" t="inlineStr">
-        <is>
-          <t>Công ty Hoàng Dung Dairy</t>
         </is>
       </c>
     </row>
@@ -5001,10 +4515,10 @@
       <c r="C10" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D10" s="93" t="n">
+      <c r="D10" s="94" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="109" t="str">
+      <c r="E10" s="110" t="str">
         <v>An Phú</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -5055,16 +4569,6 @@
       <c r="O10" s="2" t="inlineStr">
         <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>OPERATIONAL_QUANTITY_ADJUSTMENT</t>
-        </is>
-      </c>
-      <c r="Q10" s="2" t="inlineStr">
-        <is>
-          <t>An Phú</t>
         </is>
       </c>
     </row>
@@ -5076,10 +4580,10 @@
       <c r="C11" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D11" s="93" t="n">
+      <c r="D11" s="94" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="109" t="str">
+      <c r="E11" s="110" t="str">
         <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -5130,16 +4634,6 @@
       <c r="O11" s="2" t="inlineStr">
         <is>
           <t>3</t>
-        </is>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q11" s="2" t="inlineStr">
-        <is>
-          <t>Nông sản Bình Minh - giao bếp trường mỗi sáng</t>
         </is>
       </c>
     </row>
@@ -5151,10 +4645,10 @@
       <c r="C12" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D12" s="93" t="n">
+      <c r="D12" s="94" t="n">
         <v>7</v>
       </c>
-      <c r="E12" s="109" t="str">
+      <c r="E12" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -5205,16 +4699,6 @@
       <c r="O12" s="2" t="inlineStr">
         <is>
           <t>7</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q12" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -5226,10 +4710,10 @@
       <c r="C13" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D13" s="79" t="n">
+      <c r="D13" s="80" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E13" s="109" t="str">
+      <c r="E13" s="110" t="str">
         <v>Tân Thành</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -5280,16 +4764,6 @@
       <c r="O13" s="2" t="inlineStr">
         <is>
           <t>1.234567</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q13" s="2" t="inlineStr">
-        <is>
-          <t>Tân Thành</t>
         </is>
       </c>
     </row>
@@ -5301,10 +4775,10 @@
       <c r="C14" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D14" s="79" t="n">
+      <c r="D14" s="80" t="n">
         <v>0.5</v>
       </c>
-      <c r="E14" s="109" t="str">
+      <c r="E14" s="110" t="str">
         <v>Chợ A</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -5355,16 +4829,6 @@
       <c r="O14" s="2" t="inlineStr">
         <is>
           <t>0.5</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q14" s="2" t="inlineStr">
-        <is>
-          <t>Chợ A</t>
         </is>
       </c>
     </row>
@@ -5376,10 +4840,10 @@
       <c r="C15" s="25" t="str">
         <v>Kg</v>
       </c>
-      <c r="D15" s="137" t="n">
+      <c r="D15" s="138" t="n">
         <v>25</v>
       </c>
-      <c r="E15" s="113" t="str">
+      <c r="E15" s="114" t="str">
         <v>An Phú</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -5430,16 +4894,6 @@
       <c r="O15" s="2" t="inlineStr">
         <is>
           <t>25</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>PROPOSAL_ACCEPTED</t>
-        </is>
-      </c>
-      <c r="Q15" s="2" t="inlineStr">
-        <is>
-          <t>An Phú</t>
         </is>
       </c>
     </row>
@@ -5462,130 +4916,535 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="39" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="6.5" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="10.5" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <col min="6" max="15" width="1" customWidth="1" hidden="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="29" customHeight="1">
+      <c r="A1" s="4" t="str">
+        <v>Thứ Tư (22/04/2026)</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+    </row>
+    <row r="2" ht="5" customHeight="1">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+    </row>
+    <row r="3" ht="29" customHeight="1">
+      <c r="A3" s="42" t="str">
+        <v>TRƯỜNG</v>
+      </c>
+      <c r="B3" s="43" t="str">
+        <v>THÀNH PHẦN</v>
+      </c>
+      <c r="C3" s="43" t="str">
+        <v>ĐVT</v>
+      </c>
+      <c r="D3" s="43" t="str">
+        <v>SỐ LƯỢNG</v>
+      </c>
+      <c r="E3" s="44" t="str">
+        <v>GHI CHÚ</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>__workbook_marker</v>
+      </c>
+      <c r="G3" s="2" t="str">
+        <v>__line_id</v>
+      </c>
+      <c r="H3" s="2" t="str">
+        <v>__revision_id</v>
+      </c>
+      <c r="I3" s="2" t="str">
+        <v>__decision_id</v>
+      </c>
+      <c r="J3" s="2" t="str">
+        <v>__service_date</v>
+      </c>
+      <c r="K3" s="2" t="str">
+        <v>__school_id</v>
+      </c>
+      <c r="L3" s="2" t="str">
+        <v>__location_id</v>
+      </c>
+      <c r="M3" s="2" t="str">
+        <v>__ingredient_id</v>
+      </c>
+      <c r="N3" s="2" t="str">
+        <v>__unit_id</v>
+      </c>
+      <c r="O3" s="2" t="str">
+        <v>__exported_quantity</v>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="28" t="str">
+        <v>Tân Định
+Điểm giao: Bếp chính</v>
+      </c>
+      <c r="B4" s="18" t="str">
+        <v>Ớt hiểm đỏ</v>
+      </c>
+      <c r="C4" s="19" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D4" s="88" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E4" s="106" t="str">
+        <v>Công ty Hoàng Dung Dairy</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000421</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000809</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000078</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000dc</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000190</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="28" t="str">
+        <v>Tân Định
+Điểm giao: Bếp phụ</v>
+      </c>
+      <c r="B5" s="18" t="str">
+        <v>Tỏi</v>
+      </c>
+      <c r="C5" s="19" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D5" s="140" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="106" t="str">
+        <v>An Phú</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000422</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000080a</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000bf2</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000078</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000384</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000191</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="32" t="str"/>
+      <c r="B6" s="24" t="str">
+        <v>Cà rốt</v>
+      </c>
+      <c r="C6" s="25" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D6" s="138" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="114" t="str">
+        <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000423</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000080b</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000078</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000384</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000192</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" formatCells="1" formatColumns="1" formatRows="1" insertColumns="1" insertRows="1" insertHyperlinks="1" deleteColumns="1" deleteRows="1" sort="1" autoFilter="0" pivotTables="1" selectLockedCells="0" selectUnlockedCells="0" password="FB3B"/>
+  <mergeCells>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.28" right="0.28" top="0.35" bottom="0.35" header="0.12" footer="0.12"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddFooter>&amp;RTrang &amp;P / &amp;N</oddFooter>
+  </headerFooter>
+  <rowBreaks count="0" manualBreakCount="0"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="42" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="42" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="42" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="46" t="inlineStr">
+      <c r="A1" s="47" t="inlineStr">
         <is>
           <t>contract_name</t>
         </is>
       </c>
-      <c r="B1" s="46" t="inlineStr">
+      <c r="B1" s="47" t="inlineStr">
         <is>
           <t>ATLAS_SHOPPING_LIST</t>
         </is>
       </c>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
     </row>
     <row r="2">
-      <c r="A2" s="46" t="inlineStr">
+      <c r="A2" s="47" t="inlineStr">
         <is>
           <t>contract_version</t>
         </is>
       </c>
-      <c r="B2" s="46" t="inlineStr">
+      <c r="B2" s="47" t="inlineStr">
         <is>
           <t>ATLAS_SHOPPING_LIST_V1</t>
         </is>
       </c>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
     </row>
     <row r="3">
-      <c r="A3" s="46" t="inlineStr">
+      <c r="A3" s="47" t="inlineStr">
         <is>
           <t>workbook_marker</t>
         </is>
       </c>
-      <c r="B3" s="46" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
+      <c r="B3" s="47" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
     </row>
     <row r="4">
-      <c r="A4" s="46" t="inlineStr">
+      <c r="A4" s="47" t="inlineStr">
         <is>
           <t>exported_at</t>
         </is>
       </c>
-      <c r="B4" s="46" t="inlineStr">
+      <c r="B4" s="47" t="inlineStr">
         <is>
           <t>2026-04-19T10:00:00.000Z</t>
         </is>
       </c>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
     </row>
     <row r="5">
-      <c r="A5" s="46" t="inlineStr">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>service_period_start</t>
         </is>
       </c>
-      <c r="B5" s="46" t="inlineStr">
+      <c r="B5" s="47" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
     </row>
     <row r="6">
-      <c r="A6" s="46" t="inlineStr">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>service_period_end</t>
         </is>
       </c>
-      <c r="B6" s="46" t="inlineStr">
+      <c r="B6" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="C6" s="47"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="47"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="47"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="47" t="inlineStr">
+        <is>
+          <t>service_date</t>
+        </is>
+      </c>
+      <c r="B8" s="47" t="inlineStr">
+        <is>
+          <t>confirmed_need_batch_id</t>
+        </is>
+      </c>
+      <c r="C8" s="47" t="inlineStr">
+        <is>
+          <t>batch_version</t>
+        </is>
+      </c>
+      <c r="D8" s="47" t="inlineStr">
+        <is>
+          <t>need_generation_run_id</t>
+        </is>
+      </c>
+      <c r="E8" s="47" t="inlineStr">
+        <is>
+          <t>release_snapshot_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B9" s="47" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000001</t>
+        </is>
+      </c>
+      <c r="C9" s="47" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D9" s="47" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000002</t>
+        </is>
+      </c>
+      <c r="E9" s="47" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000003</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="47" t="inlineStr">
         <is>
           <t>2026-04-21</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="46" t="inlineStr">
-        <is>
-          <t>confirmed_need_batch_id</t>
-        </is>
-      </c>
-      <c r="B7" s="46" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000001</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="46" t="inlineStr">
-        <is>
-          <t>batch_version</t>
-        </is>
-      </c>
-      <c r="B8" s="46" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="46" t="inlineStr">
-        <is>
-          <t>need_generation_run_id</t>
-        </is>
-      </c>
-      <c r="B9" s="46" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000002</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="46" t="inlineStr">
-        <is>
-          <t>release_snapshot_id</t>
-        </is>
-      </c>
-      <c r="B10" s="46" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000003</t>
+      <c r="B10" s="47" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000000b</t>
+        </is>
+      </c>
+      <c r="C10" s="47" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D10" s="47" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000000c</t>
+        </is>
+      </c>
+      <c r="E10" s="47" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000000d</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="47" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B11" s="47" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000015</t>
+        </is>
+      </c>
+      <c r="C11" s="47" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D11" s="47" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000016</t>
+        </is>
+      </c>
+      <c r="E11" s="47" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000017</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(atlas): calibrate Shopping List XLSX print scale
</commit_message>
<xml_diff>
--- a/docs/xlsx/examples/atlas-shopping-list-v1-example.xlsx
+++ b/docs/xlsx/examples/atlas-shopping-list-v1-example.xlsx
@@ -29,10 +29,21 @@
     <numFmt numFmtId="200" formatCode="0.######"/>
     <numFmt numFmtId="201" formatCode="0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
     </font>
     <font>
       <sz val="14"/>
@@ -41,24 +52,7 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
+      <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
     </font>
@@ -356,34 +350,34 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="201" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -392,7 +386,7 @@
     <xf numFmtId="201" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -669,83 +663,83 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -765,10 +759,10 @@
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1048,15 +1042,15 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="26" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="39" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="6.5" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="10.5" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="7" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="25" hidden="0" customWidth="1"/>
     <col min="6" max="15" width="1" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="29" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="4" t="str">
         <v>Thứ Hai (20/04/2026)</v>
       </c>
@@ -1092,7 +1086,7 @@
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
     </row>
-    <row r="3" ht="29" customHeight="1">
+    <row r="3" ht="33" customHeight="1">
       <c r="A3" s="42" t="str">
         <v>TRƯỜNG</v>
       </c>
@@ -1139,7 +1133,7 @@
         <v>__exported_quantity</v>
       </c>
     </row>
-    <row r="4" ht="34" customHeight="1">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="28" t="str">
         <v>Trường Nguyễn Du - Cơ sở phía Đông</v>
       </c>
@@ -1206,7 +1200,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5" ht="29" customHeight="1">
       <c r="A5" s="30" t="str"/>
       <c r="B5" s="14" t="str">
         <v>Tỏi</v>
@@ -1271,7 +1265,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="29" customHeight="1">
       <c r="A6" s="30" t="str"/>
       <c r="B6" s="14" t="str">
         <v>Cà rốt</v>
@@ -1336,7 +1330,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1">
+    <row r="7" ht="29" customHeight="1">
       <c r="A7" s="30" t="str"/>
       <c r="B7" s="14" t="str">
         <v>Cải ngọt</v>
@@ -1401,7 +1395,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="34" customHeight="1">
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="30" t="str"/>
       <c r="B8" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
@@ -1466,7 +1460,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1">
+    <row r="9" ht="29" customHeight="1">
       <c r="A9" s="30" t="str"/>
       <c r="B9" s="14" t="str">
         <v>Hành lá</v>
@@ -1531,7 +1525,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
+    <row r="10" ht="29" customHeight="1">
       <c r="A10" s="30" t="str"/>
       <c r="B10" s="14" t="str">
         <v>Gạo tẻ</v>
@@ -1596,7 +1590,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1">
+    <row r="11" ht="29" customHeight="1">
       <c r="A11" s="30" t="str"/>
       <c r="B11" s="14" t="str">
         <v>Thịt heo nạc</v>
@@ -1659,7 +1653,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1">
+    <row r="12" ht="29" customHeight="1">
       <c r="A12" s="30" t="str"/>
       <c r="B12" s="14" t="str">
         <v>Trứng gà</v>
@@ -1724,7 +1718,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1">
+    <row r="13" ht="29" customHeight="1">
       <c r="A13" s="30" t="str"/>
       <c r="B13" s="14" t="str">
         <v>Dầu ăn</v>
@@ -1789,7 +1783,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1">
+    <row r="14" ht="29" customHeight="1">
       <c r="A14" s="30" t="str"/>
       <c r="B14" s="14" t="str">
         <v>Muối</v>
@@ -1854,7 +1848,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
+    <row r="15" ht="29" customHeight="1">
       <c r="A15" s="30" t="str"/>
       <c r="B15" s="14" t="str">
         <v>Nước mắm</v>
@@ -1917,7 +1911,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
+    <row r="16" ht="29" customHeight="1">
       <c r="A16" s="30" t="str"/>
       <c r="B16" s="14" t="str">
         <v>Rau ngót</v>
@@ -1982,7 +1976,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
+    <row r="17" ht="29" customHeight="1">
       <c r="A17" s="30" t="str"/>
       <c r="B17" s="14" t="str">
         <v>Bí đỏ</v>
@@ -2047,7 +2041,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="26" customHeight="1">
+    <row r="18" ht="31" customHeight="1">
       <c r="A18" s="28" t="str">
         <v>Tân Định</v>
       </c>
@@ -2114,7 +2108,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1">
+    <row r="19" ht="29" customHeight="1">
       <c r="A19" s="30" t="str"/>
       <c r="B19" s="14" t="str">
         <v>Tỏi</v>
@@ -2179,7 +2173,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1">
+    <row r="20" ht="29" customHeight="1">
       <c r="A20" s="30" t="str"/>
       <c r="B20" s="14" t="str">
         <v>Cà rốt</v>
@@ -2244,7 +2238,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1">
+    <row r="21" ht="29" customHeight="1">
       <c r="A21" s="30" t="str"/>
       <c r="B21" s="14" t="str">
         <v>Cải ngọt</v>
@@ -2309,7 +2303,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="34" customHeight="1">
+    <row r="22" ht="42" customHeight="1">
       <c r="A22" s="30" t="str"/>
       <c r="B22" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
@@ -2374,7 +2368,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="26" customHeight="1">
+    <row r="23" ht="31" customHeight="1">
       <c r="A23" s="28" t="str">
         <v>Tân Bình</v>
       </c>
@@ -2441,7 +2435,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="24" customHeight="1">
+    <row r="24" ht="29" customHeight="1">
       <c r="A24" s="30" t="str"/>
       <c r="B24" s="14" t="str">
         <v>Tỏi</v>
@@ -2506,7 +2500,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
+    <row r="25" ht="29" customHeight="1">
       <c r="A25" s="30" t="str"/>
       <c r="B25" s="14" t="str">
         <v>Cà rốt</v>
@@ -2571,8 +2565,12 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="30" t="str"/>
+    <row r="26" ht="31" customHeight="1">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>Tân Bình (tiếp)</t>
+        </is>
+      </c>
       <c r="B26" s="14" t="str">
         <v>Cải ngọt</v>
       </c>
@@ -2636,7 +2634,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="34" customHeight="1">
+    <row r="27" ht="42" customHeight="1">
       <c r="A27" s="30" t="str"/>
       <c r="B27" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
@@ -2701,7 +2699,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="24" customHeight="1">
+    <row r="28" ht="29" customHeight="1">
       <c r="A28" s="30" t="str"/>
       <c r="B28" s="14" t="str">
         <v>Hành lá</v>
@@ -2766,7 +2764,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="24" customHeight="1">
+    <row r="29" ht="29" customHeight="1">
       <c r="A29" s="30" t="str"/>
       <c r="B29" s="14" t="str">
         <v>Gạo tẻ</v>
@@ -2831,7 +2829,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="24" customHeight="1">
+    <row r="30" ht="29" customHeight="1">
       <c r="A30" s="30" t="str"/>
       <c r="B30" s="14" t="str">
         <v>Thịt heo nạc</v>
@@ -2894,7 +2892,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="24" customHeight="1">
+    <row r="31" ht="29" customHeight="1">
       <c r="A31" s="30" t="str"/>
       <c r="B31" s="14" t="str">
         <v>Trứng gà</v>
@@ -2959,12 +2957,8 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="26" customHeight="1">
-      <c r="A32" s="28" t="inlineStr">
-        <is>
-          <t>Tân Bình (tiếp)</t>
-        </is>
-      </c>
+    <row r="32" ht="29" customHeight="1">
+      <c r="A32" s="30" t="str"/>
       <c r="B32" s="14" t="str">
         <v>Dầu ăn</v>
       </c>
@@ -3028,7 +3022,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="24" customHeight="1">
+    <row r="33" ht="29" customHeight="1">
       <c r="A33" s="30" t="str"/>
       <c r="B33" s="14" t="str">
         <v>Muối</v>
@@ -3093,7 +3087,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="24" customHeight="1">
+    <row r="34" ht="29" customHeight="1">
       <c r="A34" s="30" t="str"/>
       <c r="B34" s="14" t="str">
         <v>Nước mắm</v>
@@ -3156,7 +3150,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="24" customHeight="1">
+    <row r="35" ht="29" customHeight="1">
       <c r="A35" s="30" t="str"/>
       <c r="B35" s="14" t="str">
         <v>Rau ngót</v>
@@ -3221,7 +3215,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="24" customHeight="1">
+    <row r="36" ht="29" customHeight="1">
       <c r="A36" s="30" t="str"/>
       <c r="B36" s="14" t="str">
         <v>Bí đỏ</v>
@@ -3286,7 +3280,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="24" customHeight="1">
+    <row r="37" ht="29" customHeight="1">
       <c r="A37" s="30" t="str"/>
       <c r="B37" s="14" t="str">
         <v>Khoai tây</v>
@@ -3351,7 +3345,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="24" customHeight="1">
+    <row r="38" ht="29" customHeight="1">
       <c r="A38" s="30" t="str"/>
       <c r="B38" s="14" t="str">
         <v>Cà chua</v>
@@ -3414,7 +3408,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="24" customHeight="1">
+    <row r="39" ht="29" customHeight="1">
       <c r="A39" s="30" t="str"/>
       <c r="B39" s="14" t="str">
         <v>Cần ta</v>
@@ -3479,7 +3473,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="24" customHeight="1">
+    <row r="40" ht="29" customHeight="1">
       <c r="A40" s="30" t="str"/>
       <c r="B40" s="14" t="str">
         <v>Dưa leo</v>
@@ -3544,7 +3538,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="24" customHeight="1">
+    <row r="41" ht="29" customHeight="1">
       <c r="A41" s="30" t="str"/>
       <c r="B41" s="14" t="str">
         <v>Bắp cải</v>
@@ -3609,7 +3603,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="24" customHeight="1">
+    <row r="42" ht="29" customHeight="1">
       <c r="A42" s="30" t="str"/>
       <c r="B42" s="14" t="str">
         <v>Đậu cô ve</v>
@@ -3672,7 +3666,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="24" customHeight="1">
+    <row r="43" ht="29" customHeight="1">
       <c r="A43" s="30" t="str"/>
       <c r="B43" s="14" t="str">
         <v>Su su</v>
@@ -3737,7 +3731,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="24" customHeight="1">
+    <row r="44" ht="29" customHeight="1">
       <c r="A44" s="30" t="str"/>
       <c r="B44" s="14" t="str">
         <v>Củ cải trắng</v>
@@ -3802,7 +3796,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="24" customHeight="1">
+    <row r="45" ht="29" customHeight="1">
       <c r="A45" s="30" t="str"/>
       <c r="B45" s="14" t="str">
         <v>Nấm rơm</v>
@@ -3867,7 +3861,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="24" customHeight="1">
+    <row r="46" ht="29" customHeight="1">
       <c r="A46" s="30" t="str"/>
       <c r="B46" s="14" t="str">
         <v>Sữa chua ăn</v>
@@ -3930,7 +3924,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="24" customHeight="1">
+    <row r="47" ht="29" customHeight="1">
       <c r="A47" s="32" t="str"/>
       <c r="B47" s="24" t="str">
         <v>Thịt gà phi lê</v>
@@ -4007,7 +4001,7 @@
     <oddFooter>&amp;RTrang &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="31" min="0" max="16383" man="1"/>
+    <brk id="25" min="0" max="16383" man="1"/>
   </rowBreaks>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -4022,15 +4016,15 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="26" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="39" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="6.5" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="10.5" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="7" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="25" hidden="0" customWidth="1"/>
     <col min="6" max="15" width="1" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="29" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="4" t="str">
         <v>Thứ Ba (21/04/2026)</v>
       </c>
@@ -4066,7 +4060,7 @@
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
     </row>
-    <row r="3" ht="29" customHeight="1">
+    <row r="3" ht="33" customHeight="1">
       <c r="A3" s="42" t="str">
         <v>TRƯỜNG</v>
       </c>
@@ -4113,7 +4107,7 @@
         <v>__exported_quantity</v>
       </c>
     </row>
-    <row r="4" ht="26" customHeight="1">
+    <row r="4" ht="31" customHeight="1">
       <c r="A4" s="28" t="str">
         <v>Tân Định</v>
       </c>
@@ -4180,7 +4174,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5" ht="29" customHeight="1">
       <c r="A5" s="30" t="str"/>
       <c r="B5" s="14" t="str">
         <v>Tỏi</v>
@@ -4245,7 +4239,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="29" customHeight="1">
       <c r="A6" s="30" t="str"/>
       <c r="B6" s="14" t="str">
         <v>Cà rốt</v>
@@ -4310,7 +4304,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1">
+    <row r="7" ht="29" customHeight="1">
       <c r="A7" s="30" t="str"/>
       <c r="B7" s="14" t="str">
         <v>Cải ngọt</v>
@@ -4375,7 +4369,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="34" customHeight="1">
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="30" t="str"/>
       <c r="B8" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
@@ -4440,7 +4434,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="26" customHeight="1">
+    <row r="9" ht="31" customHeight="1">
       <c r="A9" s="28" t="str">
         <v>Tân Bình</v>
       </c>
@@ -4507,7 +4501,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
+    <row r="10" ht="29" customHeight="1">
       <c r="A10" s="30" t="str"/>
       <c r="B10" s="14" t="str">
         <v>Tỏi</v>
@@ -4572,7 +4566,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1">
+    <row r="11" ht="29" customHeight="1">
       <c r="A11" s="30" t="str"/>
       <c r="B11" s="14" t="str">
         <v>Cà rốt</v>
@@ -4637,7 +4631,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1">
+    <row r="12" ht="29" customHeight="1">
       <c r="A12" s="30" t="str"/>
       <c r="B12" s="14" t="str">
         <v>Cải ngọt</v>
@@ -4702,7 +4696,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="34" customHeight="1">
+    <row r="13" ht="42" customHeight="1">
       <c r="A13" s="30" t="str"/>
       <c r="B13" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
@@ -4767,7 +4761,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1">
+    <row r="14" ht="29" customHeight="1">
       <c r="A14" s="30" t="str"/>
       <c r="B14" s="14" t="str">
         <v>Hành lá</v>
@@ -4832,7 +4826,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
+    <row r="15" ht="29" customHeight="1">
       <c r="A15" s="32" t="str"/>
       <c r="B15" s="24" t="str">
         <v>Gạo tẻ</v>
@@ -4922,15 +4916,15 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="26" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="39" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="6.5" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="10.5" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="7" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="25" hidden="0" customWidth="1"/>
     <col min="6" max="15" width="1" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="29" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="4" t="str">
         <v>Thứ Tư (22/04/2026)</v>
       </c>
@@ -4966,7 +4960,7 @@
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
     </row>
-    <row r="3" ht="29" customHeight="1">
+    <row r="3" ht="33" customHeight="1">
       <c r="A3" s="42" t="str">
         <v>TRƯỜNG</v>
       </c>
@@ -5013,7 +5007,7 @@
         <v>__exported_quantity</v>
       </c>
     </row>
-    <row r="4" ht="34" customHeight="1">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="28" t="str">
         <v>Tân Định
 Điểm giao: Bếp chính</v>
@@ -5081,7 +5075,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="28" t="str">
         <v>Tân Định
 Điểm giao: Bếp phụ</v>
@@ -5149,7 +5143,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="29" customHeight="1">
       <c r="A6" s="32" t="str"/>
       <c r="B6" s="24" t="str">
         <v>Cà rốt</v>

</xml_diff>

<commit_message>
docs(atlas): give Shopping List notes print clearance
</commit_message>
<xml_diff>
--- a/docs/xlsx/examples/atlas-shopping-list-v1-example.xlsx
+++ b/docs/xlsx/examples/atlas-shopping-list-v1-example.xlsx
@@ -1133,7 +1133,7 @@
         <v>__exported_quantity</v>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="44" customHeight="1">
       <c r="A4" s="28" t="str">
         <v>Trường Nguyễn Du - Cơ sở phía Đông</v>
       </c>
@@ -1200,7 +1200,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="29" customHeight="1">
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="30" t="str"/>
       <c r="B5" s="14" t="str">
         <v>Tỏi</v>
@@ -1265,7 +1265,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="29" customHeight="1">
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="30" t="str"/>
       <c r="B6" s="14" t="str">
         <v>Cà rốt</v>
@@ -1330,7 +1330,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="29" customHeight="1">
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="30" t="str"/>
       <c r="B7" s="14" t="str">
         <v>Cải ngọt</v>
@@ -1395,7 +1395,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
+    <row r="8" ht="44" customHeight="1">
       <c r="A8" s="30" t="str"/>
       <c r="B8" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="29" customHeight="1">
+    <row r="9" ht="32" customHeight="1">
       <c r="A9" s="30" t="str"/>
       <c r="B9" s="14" t="str">
         <v>Hành lá</v>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="29" customHeight="1">
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="30" t="str"/>
       <c r="B10" s="14" t="str">
         <v>Gạo tẻ</v>
@@ -1590,7 +1590,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="29" customHeight="1">
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="30" t="str"/>
       <c r="B11" s="14" t="str">
         <v>Thịt heo nạc</v>
@@ -1653,7 +1653,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="29" customHeight="1">
+    <row r="12" ht="32" customHeight="1">
       <c r="A12" s="30" t="str"/>
       <c r="B12" s="14" t="str">
         <v>Trứng gà</v>
@@ -1718,7 +1718,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="29" customHeight="1">
+    <row r="13" ht="32" customHeight="1">
       <c r="A13" s="30" t="str"/>
       <c r="B13" s="14" t="str">
         <v>Dầu ăn</v>
@@ -1783,7 +1783,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="29" customHeight="1">
+    <row r="14" ht="32" customHeight="1">
       <c r="A14" s="30" t="str"/>
       <c r="B14" s="14" t="str">
         <v>Muối</v>
@@ -1848,7 +1848,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="29" customHeight="1">
+    <row r="15" ht="32" customHeight="1">
       <c r="A15" s="30" t="str"/>
       <c r="B15" s="14" t="str">
         <v>Nước mắm</v>
@@ -1911,7 +1911,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="29" customHeight="1">
+    <row r="16" ht="32" customHeight="1">
       <c r="A16" s="30" t="str"/>
       <c r="B16" s="14" t="str">
         <v>Rau ngót</v>
@@ -1976,7 +1976,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="29" customHeight="1">
+    <row r="17" ht="32" customHeight="1">
       <c r="A17" s="30" t="str"/>
       <c r="B17" s="14" t="str">
         <v>Bí đỏ</v>
@@ -2041,7 +2041,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="31" customHeight="1">
+    <row r="18" ht="34" customHeight="1">
       <c r="A18" s="28" t="str">
         <v>Tân Định</v>
       </c>
@@ -2108,7 +2108,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="29" customHeight="1">
+    <row r="19" ht="32" customHeight="1">
       <c r="A19" s="30" t="str"/>
       <c r="B19" s="14" t="str">
         <v>Tỏi</v>
@@ -2173,7 +2173,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="29" customHeight="1">
+    <row r="20" ht="32" customHeight="1">
       <c r="A20" s="30" t="str"/>
       <c r="B20" s="14" t="str">
         <v>Cà rốt</v>
@@ -2238,7 +2238,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="29" customHeight="1">
+    <row r="21" ht="32" customHeight="1">
       <c r="A21" s="30" t="str"/>
       <c r="B21" s="14" t="str">
         <v>Cải ngọt</v>
@@ -2303,7 +2303,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="42" customHeight="1">
+    <row r="22" ht="44" customHeight="1">
       <c r="A22" s="30" t="str"/>
       <c r="B22" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
@@ -2368,7 +2368,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="31" customHeight="1">
+    <row r="23" ht="34" customHeight="1">
       <c r="A23" s="28" t="str">
         <v>Tân Bình</v>
       </c>
@@ -2435,7 +2435,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="29" customHeight="1">
+    <row r="24" ht="32" customHeight="1">
       <c r="A24" s="30" t="str"/>
       <c r="B24" s="14" t="str">
         <v>Tỏi</v>
@@ -2500,7 +2500,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="29" customHeight="1">
+    <row r="25" ht="32" customHeight="1">
       <c r="A25" s="30" t="str"/>
       <c r="B25" s="14" t="str">
         <v>Cà rốt</v>
@@ -2565,7 +2565,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="31" customHeight="1">
+    <row r="26" ht="34" customHeight="1">
       <c r="A26" s="28" t="inlineStr">
         <is>
           <t>Tân Bình (tiếp)</t>
@@ -2634,7 +2634,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="42" customHeight="1">
+    <row r="27" ht="44" customHeight="1">
       <c r="A27" s="30" t="str"/>
       <c r="B27" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
@@ -2699,7 +2699,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="29" customHeight="1">
+    <row r="28" ht="32" customHeight="1">
       <c r="A28" s="30" t="str"/>
       <c r="B28" s="14" t="str">
         <v>Hành lá</v>
@@ -2764,7 +2764,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="29" customHeight="1">
+    <row r="29" ht="32" customHeight="1">
       <c r="A29" s="30" t="str"/>
       <c r="B29" s="14" t="str">
         <v>Gạo tẻ</v>
@@ -2829,7 +2829,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="29" customHeight="1">
+    <row r="30" ht="32" customHeight="1">
       <c r="A30" s="30" t="str"/>
       <c r="B30" s="14" t="str">
         <v>Thịt heo nạc</v>
@@ -2892,7 +2892,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="29" customHeight="1">
+    <row r="31" ht="32" customHeight="1">
       <c r="A31" s="30" t="str"/>
       <c r="B31" s="14" t="str">
         <v>Trứng gà</v>
@@ -2957,7 +2957,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="29" customHeight="1">
+    <row r="32" ht="32" customHeight="1">
       <c r="A32" s="30" t="str"/>
       <c r="B32" s="14" t="str">
         <v>Dầu ăn</v>
@@ -3022,7 +3022,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="29" customHeight="1">
+    <row r="33" ht="32" customHeight="1">
       <c r="A33" s="30" t="str"/>
       <c r="B33" s="14" t="str">
         <v>Muối</v>
@@ -3087,7 +3087,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="29" customHeight="1">
+    <row r="34" ht="32" customHeight="1">
       <c r="A34" s="30" t="str"/>
       <c r="B34" s="14" t="str">
         <v>Nước mắm</v>
@@ -3150,7 +3150,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="29" customHeight="1">
+    <row r="35" ht="32" customHeight="1">
       <c r="A35" s="30" t="str"/>
       <c r="B35" s="14" t="str">
         <v>Rau ngót</v>
@@ -3215,7 +3215,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="29" customHeight="1">
+    <row r="36" ht="32" customHeight="1">
       <c r="A36" s="30" t="str"/>
       <c r="B36" s="14" t="str">
         <v>Bí đỏ</v>
@@ -3280,7 +3280,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="29" customHeight="1">
+    <row r="37" ht="32" customHeight="1">
       <c r="A37" s="30" t="str"/>
       <c r="B37" s="14" t="str">
         <v>Khoai tây</v>
@@ -3345,7 +3345,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="29" customHeight="1">
+    <row r="38" ht="32" customHeight="1">
       <c r="A38" s="30" t="str"/>
       <c r="B38" s="14" t="str">
         <v>Cà chua</v>
@@ -3408,7 +3408,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="29" customHeight="1">
+    <row r="39" ht="32" customHeight="1">
       <c r="A39" s="30" t="str"/>
       <c r="B39" s="14" t="str">
         <v>Cần ta</v>
@@ -3473,7 +3473,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="29" customHeight="1">
+    <row r="40" ht="32" customHeight="1">
       <c r="A40" s="30" t="str"/>
       <c r="B40" s="14" t="str">
         <v>Dưa leo</v>
@@ -3538,7 +3538,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="29" customHeight="1">
+    <row r="41" ht="32" customHeight="1">
       <c r="A41" s="30" t="str"/>
       <c r="B41" s="14" t="str">
         <v>Bắp cải</v>
@@ -3603,7 +3603,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="29" customHeight="1">
+    <row r="42" ht="32" customHeight="1">
       <c r="A42" s="30" t="str"/>
       <c r="B42" s="14" t="str">
         <v>Đậu cô ve</v>
@@ -3666,7 +3666,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="29" customHeight="1">
+    <row r="43" ht="32" customHeight="1">
       <c r="A43" s="30" t="str"/>
       <c r="B43" s="14" t="str">
         <v>Su su</v>
@@ -3731,7 +3731,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="29" customHeight="1">
+    <row r="44" ht="32" customHeight="1">
       <c r="A44" s="30" t="str"/>
       <c r="B44" s="14" t="str">
         <v>Củ cải trắng</v>
@@ -3796,7 +3796,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="29" customHeight="1">
+    <row r="45" ht="32" customHeight="1">
       <c r="A45" s="30" t="str"/>
       <c r="B45" s="14" t="str">
         <v>Nấm rơm</v>
@@ -3861,7 +3861,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="29" customHeight="1">
+    <row r="46" ht="32" customHeight="1">
       <c r="A46" s="30" t="str"/>
       <c r="B46" s="14" t="str">
         <v>Sữa chua ăn</v>
@@ -3924,7 +3924,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="29" customHeight="1">
+    <row r="47" ht="32" customHeight="1">
       <c r="A47" s="32" t="str"/>
       <c r="B47" s="24" t="str">
         <v>Thịt gà phi lê</v>
@@ -4107,7 +4107,7 @@
         <v>__exported_quantity</v>
       </c>
     </row>
-    <row r="4" ht="31" customHeight="1">
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="28" t="str">
         <v>Tân Định</v>
       </c>
@@ -4174,7 +4174,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="29" customHeight="1">
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="30" t="str"/>
       <c r="B5" s="14" t="str">
         <v>Tỏi</v>
@@ -4239,7 +4239,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="29" customHeight="1">
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="30" t="str"/>
       <c r="B6" s="14" t="str">
         <v>Cà rốt</v>
@@ -4304,7 +4304,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="29" customHeight="1">
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="30" t="str"/>
       <c r="B7" s="14" t="str">
         <v>Cải ngọt</v>
@@ -4369,7 +4369,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
+    <row r="8" ht="44" customHeight="1">
       <c r="A8" s="30" t="str"/>
       <c r="B8" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
@@ -4434,7 +4434,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="31" customHeight="1">
+    <row r="9" ht="34" customHeight="1">
       <c r="A9" s="28" t="str">
         <v>Tân Bình</v>
       </c>
@@ -4501,7 +4501,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="29" customHeight="1">
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="30" t="str"/>
       <c r="B10" s="14" t="str">
         <v>Tỏi</v>
@@ -4566,7 +4566,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="29" customHeight="1">
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="30" t="str"/>
       <c r="B11" s="14" t="str">
         <v>Cà rốt</v>
@@ -4631,7 +4631,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="29" customHeight="1">
+    <row r="12" ht="32" customHeight="1">
       <c r="A12" s="30" t="str"/>
       <c r="B12" s="14" t="str">
         <v>Cải ngọt</v>
@@ -4696,7 +4696,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="42" customHeight="1">
+    <row r="13" ht="44" customHeight="1">
       <c r="A13" s="30" t="str"/>
       <c r="B13" s="14" t="str">
         <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
@@ -4761,7 +4761,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="29" customHeight="1">
+    <row r="14" ht="32" customHeight="1">
       <c r="A14" s="30" t="str"/>
       <c r="B14" s="14" t="str">
         <v>Hành lá</v>
@@ -4826,7 +4826,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="29" customHeight="1">
+    <row r="15" ht="32" customHeight="1">
       <c r="A15" s="32" t="str"/>
       <c r="B15" s="24" t="str">
         <v>Gạo tẻ</v>
@@ -5007,7 +5007,7 @@
         <v>__exported_quantity</v>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="44" customHeight="1">
       <c r="A4" s="28" t="str">
         <v>Tân Định
 Điểm giao: Bếp chính</v>
@@ -5075,7 +5075,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="44" customHeight="1">
       <c r="A5" s="28" t="str">
         <v>Tân Định
 Điểm giao: Bếp phụ</v>
@@ -5143,7 +5143,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="29" customHeight="1">
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="32" t="str"/>
       <c r="B6" s="24" t="str">
         <v>Cà rốt</v>

</xml_diff>

<commit_message>
docs(atlas): calibrate XLSX print certification envelope
</commit_message>
<xml_diff>
--- a/docs/xlsx/examples/atlas-shopping-list-v1-example.xlsx
+++ b/docs/xlsx/examples/atlas-shopping-list-v1-example.xlsx
@@ -35,7 +35,7 @@
       <name val="Carlito"/>
     </font>
     <font>
-      <sz val="16"/>
+      <sz val="18"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
     </font>
@@ -46,13 +46,13 @@
       <name val="Times New Roman"/>
     </font>
     <font>
-      <sz val="14"/>
+      <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
-      <sz val="16"/>
+      <sz val="18"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
     </font>
@@ -248,7 +248,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="144">
+  <cellXfs count="147">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -764,6 +764,15 @@
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -774,7 +783,23 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AtlasNeed_20260420" displayName="AtlasNeed_20260420" ref="A3:O47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A3:O47"/>
+  <autoFilter ref="A3:O47">
+    <filterColumn colId="0" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="1" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="2" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="3" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="4" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="5" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="6" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="7" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="8" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="9" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="10" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="11" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="12" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="13" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="14" hiddenButton="1" showButton="0"/>
+  </autoFilter>
   <tableColumns count="15">
     <tableColumn id="1" name="TRƯỜNG"/>
     <tableColumn id="2" name="THÀNH PHẦN"/>
@@ -798,7 +823,23 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AtlasNeed_20260421" displayName="AtlasNeed_20260421" ref="A3:O15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A3:O15"/>
+  <autoFilter ref="A3:O15">
+    <filterColumn colId="0" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="1" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="2" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="3" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="4" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="5" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="6" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="7" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="8" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="9" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="10" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="11" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="12" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="13" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="14" hiddenButton="1" showButton="0"/>
+  </autoFilter>
   <tableColumns count="15">
     <tableColumn id="1" name="TRƯỜNG"/>
     <tableColumn id="2" name="THÀNH PHẦN"/>
@@ -822,7 +863,23 @@
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AtlasNeed_20260422" displayName="AtlasNeed_20260422" ref="A3:O6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A3:O6"/>
+  <autoFilter ref="A3:O6">
+    <filterColumn colId="0" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="1" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="2" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="3" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="4" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="5" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="6" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="7" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="8" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="9" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="10" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="11" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="12" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="13" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="14" hiddenButton="1" showButton="0"/>
+  </autoFilter>
   <tableColumns count="15">
     <tableColumn id="1" name="TRƯỜNG"/>
     <tableColumn id="2" name="THÀNH PHẦN"/>
@@ -1038,15 +1095,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="26" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="39" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="33" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="7" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="11" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="25" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <col min="6" max="15" width="1" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
@@ -1086,14 +1143,14 @@
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
     </row>
-    <row r="3" ht="33" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="42" t="str">
         <v>TRƯỜNG</v>
       </c>
       <c r="B3" s="43" t="str">
         <v>THÀNH PHẦN</v>
       </c>
-      <c r="C3" s="43" t="str">
+      <c r="C3" s="144" t="str">
         <v>ĐVT</v>
       </c>
       <c r="D3" s="43" t="str">
@@ -1133,9 +1190,9 @@
         <v>__exported_quantity</v>
       </c>
     </row>
-    <row r="4" ht="44" customHeight="1">
+    <row r="4" ht="72" customHeight="1">
       <c r="A4" s="28" t="str">
-        <v>Trường Nguyễn Du - Cơ sở phía Đông</v>
+        <v>Trường mẫu khu vực phía đông nam</v>
       </c>
       <c r="B4" s="18" t="str">
         <v>Ớt hiểm đỏ</v>
@@ -1147,7 +1204,7 @@
         <v>0.2</v>
       </c>
       <c r="E4" s="106" t="str">
-        <v>Công ty Hoàng Dung Dairy</v>
+        <v>Kho mẫu A</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -1200,7 +1257,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="27" customHeight="1">
       <c r="A5" s="30" t="str"/>
       <c r="B5" s="14" t="str">
         <v>Tỏi</v>
@@ -1212,7 +1269,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="110" t="str">
-        <v>An Phú</v>
+        <v>Kho mẫu D</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -1265,7 +1322,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="27" customHeight="1">
       <c r="A6" s="30" t="str"/>
       <c r="B6" s="14" t="str">
         <v>Cà rốt</v>
@@ -1277,7 +1334,7 @@
         <v>3</v>
       </c>
       <c r="E6" s="110" t="str">
-        <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
+        <v>Kho mẫu B</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -1330,7 +1387,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1">
+    <row r="7" ht="27" customHeight="1">
       <c r="A7" s="30" t="str"/>
       <c r="B7" s="14" t="str">
         <v>Cải ngọt</v>
@@ -1342,7 +1399,7 @@
         <v>7</v>
       </c>
       <c r="E7" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -1395,10 +1452,10 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="44" customHeight="1">
+    <row r="8" ht="27" customHeight="1">
       <c r="A8" s="30" t="str"/>
       <c r="B8" s="14" t="str">
-        <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
+        <v>Rau mẫu</v>
       </c>
       <c r="C8" s="15" t="str">
         <v>Kg</v>
@@ -1407,7 +1464,7 @@
         <v>1.234567</v>
       </c>
       <c r="E8" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1517,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1">
+    <row r="9" ht="27" customHeight="1">
       <c r="A9" s="30" t="str"/>
       <c r="B9" s="14" t="str">
         <v>Hành lá</v>
@@ -1472,7 +1529,7 @@
         <v>0.5</v>
       </c>
       <c r="E9" s="110" t="str">
-        <v>Chợ A</v>
+        <v>Kho mẫu E</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -1525,7 +1582,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1">
+    <row r="10" ht="27" customHeight="1">
       <c r="A10" s="30" t="str"/>
       <c r="B10" s="14" t="str">
         <v>Gạo tẻ</v>
@@ -1537,7 +1594,7 @@
         <v>25</v>
       </c>
       <c r="E10" s="110" t="str">
-        <v>An Phú</v>
+        <v>Kho mẫu D</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -1590,7 +1647,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1">
+    <row r="11" ht="27" customHeight="1">
       <c r="A11" s="30" t="str"/>
       <c r="B11" s="14" t="str">
         <v>Thịt heo nạc</v>
@@ -1653,7 +1710,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1">
+    <row r="12" ht="27" customHeight="1">
       <c r="A12" s="30" t="str"/>
       <c r="B12" s="14" t="str">
         <v>Trứng gà</v>
@@ -1665,7 +1722,7 @@
         <v>60</v>
       </c>
       <c r="E12" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1718,7 +1775,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1">
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="30" t="str"/>
       <c r="B13" s="14" t="str">
         <v>Dầu ăn</v>
@@ -1730,7 +1787,7 @@
         <v>2.5</v>
       </c>
       <c r="E13" s="110" t="str">
-        <v>Chợ A</v>
+        <v>Kho mẫu E</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1783,7 +1840,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="32" customHeight="1">
+    <row r="14" ht="27" customHeight="1">
       <c r="A14" s="30" t="str"/>
       <c r="B14" s="14" t="str">
         <v>Muối</v>
@@ -1795,7 +1852,7 @@
         <v>0.5</v>
       </c>
       <c r="E14" s="110" t="str">
-        <v>Công ty Hoàng Dung Dairy</v>
+        <v>Kho mẫu A</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1848,7 +1905,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="32" customHeight="1">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="30" t="str"/>
       <c r="B15" s="14" t="str">
         <v>Nước mắm</v>
@@ -1911,7 +1968,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="32" customHeight="1">
+    <row r="16" ht="27" customHeight="1">
       <c r="A16" s="30" t="str"/>
       <c r="B16" s="14" t="str">
         <v>Rau ngót</v>
@@ -1923,7 +1980,7 @@
         <v>0.2</v>
       </c>
       <c r="E16" s="110" t="str">
-        <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
+        <v>Kho mẫu B</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1976,7 +2033,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="32" customHeight="1">
+    <row r="17" ht="27" customHeight="1">
       <c r="A17" s="30" t="str"/>
       <c r="B17" s="14" t="str">
         <v>Bí đỏ</v>
@@ -1988,7 +2045,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -2041,9 +2098,9 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="34" customHeight="1">
+    <row r="18" ht="27" customHeight="1">
       <c r="A18" s="28" t="str">
-        <v>Tân Định</v>
+        <v>Trường mẫu B</v>
       </c>
       <c r="B18" s="18" t="str">
         <v>Ớt hiểm đỏ</v>
@@ -2055,7 +2112,7 @@
         <v>0.2</v>
       </c>
       <c r="E18" s="106" t="str">
-        <v>Công ty Hoàng Dung Dairy</v>
+        <v>Kho mẫu A</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -2108,7 +2165,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="32" customHeight="1">
+    <row r="19" ht="27" customHeight="1">
       <c r="A19" s="30" t="str"/>
       <c r="B19" s="14" t="str">
         <v>Tỏi</v>
@@ -2120,7 +2177,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="110" t="str">
-        <v>An Phú</v>
+        <v>Kho mẫu D</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -2173,7 +2230,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1">
+    <row r="20" ht="27" customHeight="1">
       <c r="A20" s="30" t="str"/>
       <c r="B20" s="14" t="str">
         <v>Cà rốt</v>
@@ -2185,7 +2242,7 @@
         <v>3</v>
       </c>
       <c r="E20" s="110" t="str">
-        <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
+        <v>Kho mẫu B</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -2238,7 +2295,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="32" customHeight="1">
+    <row r="21" ht="27" customHeight="1">
       <c r="A21" s="30" t="str"/>
       <c r="B21" s="14" t="str">
         <v>Cải ngọt</v>
@@ -2250,7 +2307,7 @@
         <v>7</v>
       </c>
       <c r="E21" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -2303,10 +2360,10 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="44" customHeight="1">
+    <row r="22" ht="27" customHeight="1">
       <c r="A22" s="30" t="str"/>
       <c r="B22" s="14" t="str">
-        <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
+        <v>Rau mẫu</v>
       </c>
       <c r="C22" s="15" t="str">
         <v>Kg</v>
@@ -2315,7 +2372,7 @@
         <v>1.234567</v>
       </c>
       <c r="E22" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -2368,21 +2425,21 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="34" customHeight="1">
+    <row r="23" ht="72" customHeight="1">
       <c r="A23" s="28" t="str">
-        <v>Tân Bình</v>
+        <v>Trường mẫu C</v>
       </c>
       <c r="B23" s="18" t="str">
-        <v>Ớt hiểm đỏ</v>
+        <v>Rau củ mô phỏng theo quy cách bếp mẫu</v>
       </c>
       <c r="C23" s="19" t="str">
         <v>Kg</v>
       </c>
       <c r="D23" s="88" t="n">
-        <v>0.2</v>
+        <v>123456789.1</v>
       </c>
       <c r="E23" s="106" t="str">
-        <v>Công ty Hoàng Dung Dairy</v>
+        <v>Kho mẫu phía đông</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -2421,7 +2478,7 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>00000000-0000-0000-0000-000000000190</t>
+          <t>00000000-0000-0000-0000-0000000002bc</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -2431,11 +2488,11 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>0.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="32" customHeight="1">
+          <t>123456789.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="27" customHeight="1">
       <c r="A24" s="30" t="str"/>
       <c r="B24" s="14" t="str">
         <v>Tỏi</v>
@@ -2443,11 +2500,11 @@
       <c r="C24" s="15" t="str">
         <v>Kg</v>
       </c>
-      <c r="D24" s="94" t="n">
-        <v>1</v>
+      <c r="D24" s="80" t="n">
+        <v>1234567890.1</v>
       </c>
       <c r="E24" s="110" t="str">
-        <v>An Phú</v>
+        <v>Kho mẫu D</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -2496,14 +2553,14 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="32" customHeight="1">
+          <t>1234567890.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="72" customHeight="1">
       <c r="A25" s="30" t="str"/>
       <c r="B25" s="14" t="str">
-        <v>Cà rốt</v>
+        <v>Ớt mẫu</v>
       </c>
       <c r="C25" s="15" t="str">
         <v>Kg</v>
@@ -2512,7 +2569,7 @@
         <v>3</v>
       </c>
       <c r="E25" s="110" t="str">
-        <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
+        <v>Cơ sở thực phẩm giả lập A</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -2551,7 +2608,7 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>00000000-0000-0000-0000-000000000192</t>
+          <t>00000000-0000-0000-0000-0000000002bd</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -2565,10 +2622,10 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="34" customHeight="1">
+    <row r="26" ht="72" customHeight="1">
       <c r="A26" s="28" t="inlineStr">
         <is>
-          <t>Tân Bình (tiếp)</t>
+          <t>Trường mẫu C (tiếp)</t>
         </is>
       </c>
       <c r="B26" s="14" t="str">
@@ -2581,7 +2638,7 @@
         <v>7</v>
       </c>
       <c r="E26" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -2634,10 +2691,10 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="44" customHeight="1">
+    <row r="27" ht="27" customHeight="1">
       <c r="A27" s="30" t="str"/>
       <c r="B27" s="14" t="str">
-        <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
+        <v>Rau mẫu</v>
       </c>
       <c r="C27" s="15" t="str">
         <v>Kg</v>
@@ -2646,7 +2703,7 @@
         <v>1.234567</v>
       </c>
       <c r="E27" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -2699,7 +2756,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="32" customHeight="1">
+    <row r="28" ht="27" customHeight="1">
       <c r="A28" s="30" t="str"/>
       <c r="B28" s="14" t="str">
         <v>Hành lá</v>
@@ -2711,7 +2768,7 @@
         <v>0.5</v>
       </c>
       <c r="E28" s="110" t="str">
-        <v>Chợ A</v>
+        <v>Kho mẫu E</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -2764,7 +2821,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="32" customHeight="1">
+    <row r="29" ht="27" customHeight="1">
       <c r="A29" s="30" t="str"/>
       <c r="B29" s="14" t="str">
         <v>Gạo tẻ</v>
@@ -2776,7 +2833,7 @@
         <v>25</v>
       </c>
       <c r="E29" s="110" t="str">
-        <v>An Phú</v>
+        <v>Kho mẫu D</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -2829,7 +2886,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="32" customHeight="1">
+    <row r="30" ht="27" customHeight="1">
       <c r="A30" s="30" t="str"/>
       <c r="B30" s="14" t="str">
         <v>Thịt heo nạc</v>
@@ -2892,7 +2949,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="32" customHeight="1">
+    <row r="31" ht="27" customHeight="1">
       <c r="A31" s="30" t="str"/>
       <c r="B31" s="14" t="str">
         <v>Trứng gà</v>
@@ -2904,7 +2961,7 @@
         <v>60</v>
       </c>
       <c r="E31" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2957,7 +3014,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="32" customHeight="1">
+    <row r="32" ht="27" customHeight="1">
       <c r="A32" s="30" t="str"/>
       <c r="B32" s="14" t="str">
         <v>Dầu ăn</v>
@@ -2969,7 +3026,7 @@
         <v>2.5</v>
       </c>
       <c r="E32" s="110" t="str">
-        <v>Chợ A</v>
+        <v>Kho mẫu E</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -3022,7 +3079,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="32" customHeight="1">
+    <row r="33" ht="27" customHeight="1">
       <c r="A33" s="30" t="str"/>
       <c r="B33" s="14" t="str">
         <v>Muối</v>
@@ -3034,7 +3091,7 @@
         <v>0.5</v>
       </c>
       <c r="E33" s="110" t="str">
-        <v>Công ty Hoàng Dung Dairy</v>
+        <v>Kho mẫu A</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -3087,7 +3144,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="32" customHeight="1">
+    <row r="34" ht="27" customHeight="1">
       <c r="A34" s="30" t="str"/>
       <c r="B34" s="14" t="str">
         <v>Nước mắm</v>
@@ -3150,7 +3207,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="32" customHeight="1">
+    <row r="35" ht="27" customHeight="1">
       <c r="A35" s="30" t="str"/>
       <c r="B35" s="14" t="str">
         <v>Rau ngót</v>
@@ -3162,7 +3219,7 @@
         <v>0.2</v>
       </c>
       <c r="E35" s="110" t="str">
-        <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
+        <v>Kho mẫu B</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -3215,7 +3272,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="32" customHeight="1">
+    <row r="36" ht="27" customHeight="1">
       <c r="A36" s="30" t="str"/>
       <c r="B36" s="14" t="str">
         <v>Bí đỏ</v>
@@ -3227,7 +3284,7 @@
         <v>1</v>
       </c>
       <c r="E36" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -3280,7 +3337,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="32" customHeight="1">
+    <row r="37" ht="27" customHeight="1">
       <c r="A37" s="30" t="str"/>
       <c r="B37" s="14" t="str">
         <v>Khoai tây</v>
@@ -3292,7 +3349,7 @@
         <v>3</v>
       </c>
       <c r="E37" s="110" t="str">
-        <v>Chợ A</v>
+        <v>Kho mẫu E</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -3345,7 +3402,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="32" customHeight="1">
+    <row r="38" ht="27" customHeight="1">
       <c r="A38" s="30" t="str"/>
       <c r="B38" s="14" t="str">
         <v>Cà chua</v>
@@ -3408,7 +3465,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="32" customHeight="1">
+    <row r="39" ht="27" customHeight="1">
       <c r="A39" s="30" t="str"/>
       <c r="B39" s="14" t="str">
         <v>Cần ta</v>
@@ -3420,7 +3477,7 @@
         <v>31</v>
       </c>
       <c r="E39" s="110" t="str">
-        <v>An Phú</v>
+        <v>Kho mẫu D</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -3473,7 +3530,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="32" customHeight="1">
+    <row r="40" ht="27" customHeight="1">
       <c r="A40" s="30" t="str"/>
       <c r="B40" s="14" t="str">
         <v>Dưa leo</v>
@@ -3485,7 +3542,7 @@
         <v>0.5</v>
       </c>
       <c r="E40" s="110" t="str">
-        <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
+        <v>Kho mẫu B</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -3538,7 +3595,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="32" customHeight="1">
+    <row r="41" ht="27" customHeight="1">
       <c r="A41" s="30" t="str"/>
       <c r="B41" s="14" t="str">
         <v>Bắp cải</v>
@@ -3550,7 +3607,7 @@
         <v>25</v>
       </c>
       <c r="E41" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -3603,7 +3660,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="32" customHeight="1">
+    <row r="42" ht="27" customHeight="1">
       <c r="A42" s="30" t="str"/>
       <c r="B42" s="14" t="str">
         <v>Đậu cô ve</v>
@@ -3666,7 +3723,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="32" customHeight="1">
+    <row r="43" ht="27" customHeight="1">
       <c r="A43" s="30" t="str"/>
       <c r="B43" s="14" t="str">
         <v>Su su</v>
@@ -3678,7 +3735,7 @@
         <v>60</v>
       </c>
       <c r="E43" s="110" t="str">
-        <v>Công ty Hoàng Dung Dairy</v>
+        <v>Kho mẫu A</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -3731,7 +3788,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="32" customHeight="1">
+    <row r="44" ht="27" customHeight="1">
       <c r="A44" s="30" t="str"/>
       <c r="B44" s="14" t="str">
         <v>Củ cải trắng</v>
@@ -3743,7 +3800,7 @@
         <v>2.5</v>
       </c>
       <c r="E44" s="110" t="str">
-        <v>An Phú</v>
+        <v>Kho mẫu D</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -3796,7 +3853,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="32" customHeight="1">
+    <row r="45" ht="27" customHeight="1">
       <c r="A45" s="30" t="str"/>
       <c r="B45" s="14" t="str">
         <v>Nấm rơm</v>
@@ -3808,7 +3865,7 @@
         <v>0.5</v>
       </c>
       <c r="E45" s="110" t="str">
-        <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
+        <v>Kho mẫu B</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -3861,7 +3918,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="32" customHeight="1">
+    <row r="46" ht="27" customHeight="1">
       <c r="A46" s="30" t="str"/>
       <c r="B46" s="14" t="str">
         <v>Sữa chua ăn</v>
@@ -3924,7 +3981,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="32" customHeight="1">
+    <row r="47" ht="27" customHeight="1">
       <c r="A47" s="32" t="str"/>
       <c r="B47" s="24" t="str">
         <v>Thịt gà phi lê</v>
@@ -3936,7 +3993,7 @@
         <v>0.2</v>
       </c>
       <c r="E47" s="114" t="str">
-        <v>Chợ A</v>
+        <v>Kho mẫu E</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -3995,8 +4052,8 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.28" right="0.28" top="0.35" bottom="0.35" header="0.12" footer="0.12"/>
-  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
+  <pageMargins left="0.2" right="0.2" top="0.25" bottom="0.25" header="0.12" footer="0.12"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="95"/>
   <headerFooter>
     <oddFooter>&amp;RTrang &amp;P / &amp;N</oddFooter>
   </headerFooter>
@@ -4012,15 +4069,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="26" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="39" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="33" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="7" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="11" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="25" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <col min="6" max="15" width="1" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
@@ -4060,14 +4117,14 @@
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
     </row>
-    <row r="3" ht="33" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="42" t="str">
         <v>TRƯỜNG</v>
       </c>
       <c r="B3" s="43" t="str">
         <v>THÀNH PHẦN</v>
       </c>
-      <c r="C3" s="43" t="str">
+      <c r="C3" s="145" t="str">
         <v>ĐVT</v>
       </c>
       <c r="D3" s="43" t="str">
@@ -4107,9 +4164,9 @@
         <v>__exported_quantity</v>
       </c>
     </row>
-    <row r="4" ht="34" customHeight="1">
+    <row r="4" ht="27" customHeight="1">
       <c r="A4" s="28" t="str">
-        <v>Tân Định</v>
+        <v>Trường mẫu B</v>
       </c>
       <c r="B4" s="18" t="str">
         <v>Ớt hiểm đỏ</v>
@@ -4121,7 +4178,7 @@
         <v>0.2</v>
       </c>
       <c r="E4" s="106" t="str">
-        <v>Công ty Hoàng Dung Dairy</v>
+        <v>Kho mẫu A</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -4174,7 +4231,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="27" customHeight="1">
       <c r="A5" s="30" t="str"/>
       <c r="B5" s="14" t="str">
         <v>Tỏi</v>
@@ -4186,7 +4243,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="110" t="str">
-        <v>An Phú</v>
+        <v>Kho mẫu D</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -4239,7 +4296,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="27" customHeight="1">
       <c r="A6" s="30" t="str"/>
       <c r="B6" s="14" t="str">
         <v>Cà rốt</v>
@@ -4251,7 +4308,7 @@
         <v>3</v>
       </c>
       <c r="E6" s="110" t="str">
-        <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
+        <v>Kho mẫu B</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -4304,7 +4361,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1">
+    <row r="7" ht="27" customHeight="1">
       <c r="A7" s="30" t="str"/>
       <c r="B7" s="14" t="str">
         <v>Cải ngọt</v>
@@ -4316,7 +4373,7 @@
         <v>7</v>
       </c>
       <c r="E7" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -4369,10 +4426,10 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="44" customHeight="1">
+    <row r="8" ht="27" customHeight="1">
       <c r="A8" s="30" t="str"/>
       <c r="B8" s="14" t="str">
-        <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
+        <v>Rau mẫu</v>
       </c>
       <c r="C8" s="15" t="str">
         <v>Kg</v>
@@ -4381,7 +4438,7 @@
         <v>1.234567</v>
       </c>
       <c r="E8" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -4434,12 +4491,12 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="34" customHeight="1">
+    <row r="9" ht="72" customHeight="1">
       <c r="A9" s="28" t="str">
-        <v>Tân Bình</v>
+        <v>Trường mẫu C</v>
       </c>
       <c r="B9" s="18" t="str">
-        <v>Ớt hiểm đỏ</v>
+        <v>Rau củ mô phỏng sơ chế theo quy cách bếp số mười</v>
       </c>
       <c r="C9" s="19" t="str">
         <v>Kg</v>
@@ -4448,7 +4505,7 @@
         <v>0.2</v>
       </c>
       <c r="E9" s="106" t="str">
-        <v>Công ty Hoàng Dung Dairy</v>
+        <v>Kho</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -4487,7 +4544,7 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>00000000-0000-0000-0000-000000000190</t>
+          <t>00000000-0000-0000-0000-0000000002be</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -4501,7 +4558,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1">
+    <row r="10" ht="27" customHeight="1">
       <c r="A10" s="30" t="str"/>
       <c r="B10" s="14" t="str">
         <v>Tỏi</v>
@@ -4513,7 +4570,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="110" t="str">
-        <v>An Phú</v>
+        <v>Kho mẫu D</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4623,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1">
+    <row r="11" ht="27" customHeight="1">
       <c r="A11" s="30" t="str"/>
       <c r="B11" s="14" t="str">
         <v>Cà rốt</v>
@@ -4578,7 +4635,7 @@
         <v>3</v>
       </c>
       <c r="E11" s="110" t="str">
-        <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
+        <v>Kho mẫu B</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -4631,7 +4688,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1">
+    <row r="12" ht="27" customHeight="1">
       <c r="A12" s="30" t="str"/>
       <c r="B12" s="14" t="str">
         <v>Cải ngọt</v>
@@ -4643,7 +4700,7 @@
         <v>7</v>
       </c>
       <c r="E12" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -4696,10 +4753,10 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="44" customHeight="1">
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="30" t="str"/>
       <c r="B13" s="14" t="str">
-        <v>Đu đủ hường sơ chế, bỏ vỏ và hạt, cắt miếng theo quy cách bếp trường</v>
+        <v>Rau mẫu</v>
       </c>
       <c r="C13" s="15" t="str">
         <v>Kg</v>
@@ -4708,7 +4765,7 @@
         <v>1.234567</v>
       </c>
       <c r="E13" s="110" t="str">
-        <v>Tân Thành</v>
+        <v>Kho mẫu C</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -4761,7 +4818,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="32" customHeight="1">
+    <row r="14" ht="27" customHeight="1">
       <c r="A14" s="30" t="str"/>
       <c r="B14" s="14" t="str">
         <v>Hành lá</v>
@@ -4773,7 +4830,7 @@
         <v>0.5</v>
       </c>
       <c r="E14" s="110" t="str">
-        <v>Chợ A</v>
+        <v>Kho mẫu E</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -4826,7 +4883,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="32" customHeight="1">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="32" t="str"/>
       <c r="B15" s="24" t="str">
         <v>Gạo tẻ</v>
@@ -4838,7 +4895,7 @@
         <v>25</v>
       </c>
       <c r="E15" s="114" t="str">
-        <v>An Phú</v>
+        <v>Kho mẫu D</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -4897,8 +4954,8 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.28" right="0.28" top="0.35" bottom="0.35" header="0.12" footer="0.12"/>
-  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
+  <pageMargins left="0.2" right="0.2" top="0.25" bottom="0.25" header="0.12" footer="0.12"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="95"/>
   <headerFooter>
     <oddFooter>&amp;RTrang &amp;P / &amp;N</oddFooter>
   </headerFooter>
@@ -4912,15 +4969,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="26" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="39" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="33" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="7" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="11" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="25" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <col min="6" max="15" width="1" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
@@ -4960,14 +5017,14 @@
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
     </row>
-    <row r="3" ht="33" customHeight="1">
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="42" t="str">
         <v>TRƯỜNG</v>
       </c>
       <c r="B3" s="43" t="str">
         <v>THÀNH PHẦN</v>
       </c>
-      <c r="C3" s="43" t="str">
+      <c r="C3" s="146" t="str">
         <v>ĐVT</v>
       </c>
       <c r="D3" s="43" t="str">
@@ -5007,22 +5064,22 @@
         <v>__exported_quantity</v>
       </c>
     </row>
-    <row r="4" ht="44" customHeight="1">
+    <row r="4" ht="168" customHeight="1">
       <c r="A4" s="28" t="str">
-        <v>Tân Định
-Điểm giao: Bếp chính</v>
+        <v>Trường mẫu khu vực phía đông bắc
+Điểm giao: Bếp mô phỏng khu vực phía đông A</v>
       </c>
       <c r="B4" s="18" t="str">
-        <v>Ớt hiểm đỏ</v>
+        <v>Rau</v>
       </c>
       <c r="C4" s="19" t="str">
         <v>Kg</v>
       </c>
-      <c r="D4" s="88" t="n">
-        <v>0.2</v>
+      <c r="D4" s="140" t="n">
+        <v>1</v>
       </c>
       <c r="E4" s="106" t="str">
-        <v>Công ty Hoàng Dung Dairy</v>
+        <v>Kho</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -5051,17 +5108,17 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>00000000-0000-0000-0000-000000000078</t>
+          <t>00000000-0000-0000-0000-00000000008c</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>00000000-0000-0000-0000-0000000000dc</t>
+          <t>00000000-0000-0000-0000-0000000000f0</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>00000000-0000-0000-0000-000000000190</t>
+          <t>00000000-0000-0000-0000-0000000002bf</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -5071,14 +5128,14 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>0.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44" customHeight="1">
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="168" customHeight="1">
       <c r="A5" s="28" t="str">
-        <v>Tân Định
-Điểm giao: Bếp phụ</v>
+        <v>Trường mẫu khu vực phía đông bắc
+Điểm giao: Bếp mẫu B</v>
       </c>
       <c r="B5" s="18" t="str">
         <v>Tỏi</v>
@@ -5090,7 +5147,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="106" t="str">
-        <v>An Phú</v>
+        <v>Kho mẫu D</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -5119,12 +5176,12 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>00000000-0000-0000-0000-000000000078</t>
+          <t>00000000-0000-0000-0000-00000000008c</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>00000000-0000-0000-0000-000000000384</t>
+          <t>00000000-0000-0000-0000-0000000003ac</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -5143,7 +5200,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="27" customHeight="1">
       <c r="A6" s="32" t="str"/>
       <c r="B6" s="24" t="str">
         <v>Cà rốt</v>
@@ -5155,7 +5212,7 @@
         <v>3</v>
       </c>
       <c r="E6" s="114" t="str">
-        <v>Nông sản Bình Minh - giao bếp trường mỗi sáng</v>
+        <v>Kho mẫu B</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -5184,12 +5241,12 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>00000000-0000-0000-0000-000000000078</t>
+          <t>00000000-0000-0000-0000-00000000008c</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>00000000-0000-0000-0000-000000000384</t>
+          <t>00000000-0000-0000-0000-0000000003ac</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -5214,8 +5271,8 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.28" right="0.28" top="0.35" bottom="0.35" header="0.12" footer="0.12"/>
-  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
+  <pageMargins left="0.2" right="0.2" top="0.25" bottom="0.25" header="0.12" footer="0.12"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="95"/>
   <headerFooter>
     <oddFooter>&amp;RTrang &amp;P / &amp;N</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
docs(atlas): finalize School-only Shopping List XLSX V1
</commit_message>
<xml_diff>
--- a/docs/xlsx/examples/atlas-shopping-list-v1-example.xlsx
+++ b/docs/xlsx/examples/atlas-shopping-list-v1-example.xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="200" formatCode="0.######"/>
     <numFmt numFmtId="201" formatCode="0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -46,6 +46,11 @@
       <name val="Times New Roman"/>
     </font>
     <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
       <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
@@ -53,6 +58,12 @@
     <font>
       <b/>
       <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="17"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
     </font>
@@ -275,10 +286,13 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="0"/>
     </xf>
-    <xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="200" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="200" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -293,7 +307,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="0"/>
     </xf>
-    <xf numFmtId="200" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="200" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -305,16 +319,16 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="0"/>
     </xf>
-    <xf numFmtId="200" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="200" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="201" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="201" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -323,13 +337,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="0"/>
     </xf>
-    <xf numFmtId="200" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="200" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -350,43 +364,40 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="201" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="201" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
     </xf>
-    <xf numFmtId="201" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -463,19 +474,27 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="200" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="0"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="200" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
@@ -511,11 +530,11 @@
       <alignment horizontal="center" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="200" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="200" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
@@ -543,11 +562,11 @@
       <alignment horizontal="center" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="200" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="200" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
@@ -559,19 +578,19 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="201" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="201" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
@@ -591,11 +610,11 @@
       <alignment horizontal="center" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="200" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="200" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
@@ -607,11 +626,11 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -663,115 +682,107 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="201" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="201" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="0"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="201" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="0"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center" wrapText="0"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
@@ -1099,11 +1110,11 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="33" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="7" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="19" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="6" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="15" hidden="0" customWidth="1"/>
     <col min="6" max="15" width="1" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
@@ -1144,19 +1155,19 @@
       <c r="O2" s="2"/>
     </row>
     <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="42" t="str">
+      <c r="A3" s="43" t="str">
         <v>TRƯỜNG</v>
       </c>
-      <c r="B3" s="43" t="str">
+      <c r="B3" s="44" t="str">
         <v>THÀNH PHẦN</v>
       </c>
       <c r="C3" s="144" t="str">
         <v>ĐVT</v>
       </c>
-      <c r="D3" s="43" t="str">
+      <c r="D3" s="44" t="str">
         <v>SỐ LƯỢNG</v>
       </c>
-      <c r="E3" s="44" t="str">
+      <c r="E3" s="45" t="str">
         <v>GHI CHÚ</v>
       </c>
       <c r="F3" s="2" t="str">
@@ -1190,20 +1201,20 @@
         <v>__exported_quantity</v>
       </c>
     </row>
-    <row r="4" ht="72" customHeight="1">
-      <c r="A4" s="28" t="str">
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="29" t="str">
         <v>Trường mẫu khu vực phía đông nam</v>
       </c>
-      <c r="B4" s="18" t="str">
+      <c r="B4" s="19" t="str">
         <v>Ớt hiểm đỏ</v>
       </c>
-      <c r="C4" s="19" t="str">
+      <c r="C4" s="20" t="str">
         <v>Kg</v>
       </c>
-      <c r="D4" s="88" t="n">
+      <c r="D4" s="90" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="106" t="str">
+      <c r="E4" s="108" t="str">
         <v>Kho mẫu A</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1257,18 +1268,18 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="27" customHeight="1">
-      <c r="A5" s="30" t="str"/>
-      <c r="B5" s="14" t="str">
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="31" t="str"/>
+      <c r="B5" s="15" t="str">
         <v>Tỏi</v>
       </c>
-      <c r="C5" s="15" t="str">
+      <c r="C5" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D5" s="94" t="n">
+      <c r="D5" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="110" t="str">
+      <c r="E5" s="112" t="str">
         <v>Kho mẫu D</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1322,18 +1333,18 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="27" customHeight="1">
-      <c r="A6" s="30" t="str"/>
-      <c r="B6" s="14" t="str">
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="31" t="str"/>
+      <c r="B6" s="15" t="str">
         <v>Cà rốt</v>
       </c>
-      <c r="C6" s="15" t="str">
+      <c r="C6" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D6" s="94" t="n">
+      <c r="D6" s="96" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="110" t="str">
+      <c r="E6" s="112" t="str">
         <v>Kho mẫu B</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1387,18 +1398,18 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="27" customHeight="1">
-      <c r="A7" s="30" t="str"/>
-      <c r="B7" s="14" t="str">
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="31" t="str"/>
+      <c r="B7" s="15" t="str">
         <v>Cải ngọt</v>
       </c>
-      <c r="C7" s="15" t="str">
+      <c r="C7" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D7" s="94" t="n">
+      <c r="D7" s="96" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="110" t="str">
+      <c r="E7" s="112" t="str">
         <v>Kho mẫu C</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1452,18 +1463,18 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="27" customHeight="1">
-      <c r="A8" s="30" t="str"/>
-      <c r="B8" s="14" t="str">
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="31" t="str"/>
+      <c r="B8" s="15" t="str">
         <v>Rau mẫu</v>
       </c>
-      <c r="C8" s="15" t="str">
+      <c r="C8" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D8" s="80" t="n">
+      <c r="D8" s="82" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E8" s="110" t="str">
+      <c r="E8" s="112" t="str">
         <v>Kho mẫu C</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1517,18 +1528,18 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="27" customHeight="1">
-      <c r="A9" s="30" t="str"/>
-      <c r="B9" s="14" t="str">
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="31" t="str"/>
+      <c r="B9" s="15" t="str">
         <v>Hành lá</v>
       </c>
-      <c r="C9" s="15" t="str">
+      <c r="C9" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D9" s="80" t="n">
+      <c r="D9" s="82" t="n">
         <v>0.5</v>
       </c>
-      <c r="E9" s="110" t="str">
+      <c r="E9" s="112" t="str">
         <v>Kho mẫu E</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1582,18 +1593,18 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="27" customHeight="1">
-      <c r="A10" s="30" t="str"/>
-      <c r="B10" s="14" t="str">
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="31" t="str"/>
+      <c r="B10" s="15" t="str">
         <v>Gạo tẻ</v>
       </c>
-      <c r="C10" s="15" t="str">
+      <c r="C10" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D10" s="94" t="n">
+      <c r="D10" s="96" t="n">
         <v>25</v>
       </c>
-      <c r="E10" s="110" t="str">
+      <c r="E10" s="112" t="str">
         <v>Kho mẫu D</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1647,18 +1658,18 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="27" customHeight="1">
-      <c r="A11" s="30" t="str"/>
-      <c r="B11" s="14" t="str">
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="31" t="str"/>
+      <c r="B11" s="15" t="str">
         <v>Thịt heo nạc</v>
       </c>
-      <c r="C11" s="15" t="str">
+      <c r="C11" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D11" s="80" t="n">
+      <c r="D11" s="82" t="n">
         <v>12.5</v>
       </c>
-      <c r="E11" s="110" t="str"/>
+      <c r="E11" s="112" t="str"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -1710,18 +1721,18 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="27" customHeight="1">
-      <c r="A12" s="30" t="str"/>
-      <c r="B12" s="14" t="str">
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="31" t="str"/>
+      <c r="B12" s="15" t="str">
         <v>Trứng gà</v>
       </c>
-      <c r="C12" s="15" t="str">
+      <c r="C12" s="16" t="str">
         <v>Quả</v>
       </c>
-      <c r="D12" s="94" t="n">
+      <c r="D12" s="96" t="n">
         <v>60</v>
       </c>
-      <c r="E12" s="110" t="str">
+      <c r="E12" s="112" t="str">
         <v>Kho mẫu C</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1775,18 +1786,18 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="27" customHeight="1">
-      <c r="A13" s="30" t="str"/>
-      <c r="B13" s="14" t="str">
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="31" t="str"/>
+      <c r="B13" s="15" t="str">
         <v>Dầu ăn</v>
       </c>
-      <c r="C13" s="15" t="str">
+      <c r="C13" s="16" t="str">
         <v>Lít</v>
       </c>
-      <c r="D13" s="80" t="n">
+      <c r="D13" s="82" t="n">
         <v>2.5</v>
       </c>
-      <c r="E13" s="110" t="str">
+      <c r="E13" s="112" t="str">
         <v>Kho mẫu E</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1840,18 +1851,18 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="27" customHeight="1">
-      <c r="A14" s="30" t="str"/>
-      <c r="B14" s="14" t="str">
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="31" t="str"/>
+      <c r="B14" s="15" t="str">
         <v>Muối</v>
       </c>
-      <c r="C14" s="15" t="str">
+      <c r="C14" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D14" s="80" t="n">
+      <c r="D14" s="82" t="n">
         <v>0.5</v>
       </c>
-      <c r="E14" s="110" t="str">
+      <c r="E14" s="112" t="str">
         <v>Kho mẫu A</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1905,18 +1916,18 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="27" customHeight="1">
-      <c r="A15" s="30" t="str"/>
-      <c r="B15" s="14" t="str">
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="31" t="str"/>
+      <c r="B15" s="15" t="str">
         <v>Nước mắm</v>
       </c>
-      <c r="C15" s="15" t="str">
+      <c r="C15" s="16" t="str">
         <v>Lít</v>
       </c>
-      <c r="D15" s="94" t="n">
+      <c r="D15" s="96" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="110" t="str"/>
+      <c r="E15" s="112" t="str"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000002328</t>
@@ -1968,18 +1979,18 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="27" customHeight="1">
-      <c r="A16" s="30" t="str"/>
-      <c r="B16" s="14" t="str">
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="31" t="str"/>
+      <c r="B16" s="15" t="str">
         <v>Rau ngót</v>
       </c>
-      <c r="C16" s="15" t="str">
+      <c r="C16" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D16" s="80" t="n">
+      <c r="D16" s="82" t="n">
         <v>0.2</v>
       </c>
-      <c r="E16" s="110" t="str">
+      <c r="E16" s="112" t="str">
         <v>Kho mẫu B</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -2033,18 +2044,18 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="27" customHeight="1">
-      <c r="A17" s="30" t="str"/>
-      <c r="B17" s="14" t="str">
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="31" t="str"/>
+      <c r="B17" s="15" t="str">
         <v>Bí đỏ</v>
       </c>
-      <c r="C17" s="15" t="str">
+      <c r="C17" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D17" s="94" t="n">
+      <c r="D17" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="110" t="str">
+      <c r="E17" s="112" t="str">
         <v>Kho mẫu C</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -2098,20 +2109,20 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="27" customHeight="1">
-      <c r="A18" s="28" t="str">
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="29" t="str">
         <v>Trường mẫu B</v>
       </c>
-      <c r="B18" s="18" t="str">
+      <c r="B18" s="19" t="str">
         <v>Ớt hiểm đỏ</v>
       </c>
-      <c r="C18" s="19" t="str">
+      <c r="C18" s="20" t="str">
         <v>Kg</v>
       </c>
-      <c r="D18" s="88" t="n">
+      <c r="D18" s="90" t="n">
         <v>0.2</v>
       </c>
-      <c r="E18" s="106" t="str">
+      <c r="E18" s="108" t="str">
         <v>Kho mẫu A</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -2165,18 +2176,18 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="27" customHeight="1">
-      <c r="A19" s="30" t="str"/>
-      <c r="B19" s="14" t="str">
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="31" t="str"/>
+      <c r="B19" s="15" t="str">
         <v>Tỏi</v>
       </c>
-      <c r="C19" s="15" t="str">
+      <c r="C19" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D19" s="94" t="n">
+      <c r="D19" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="110" t="str">
+      <c r="E19" s="112" t="str">
         <v>Kho mẫu D</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -2230,18 +2241,18 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="27" customHeight="1">
-      <c r="A20" s="30" t="str"/>
-      <c r="B20" s="14" t="str">
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="31" t="str"/>
+      <c r="B20" s="15" t="str">
         <v>Cà rốt</v>
       </c>
-      <c r="C20" s="15" t="str">
+      <c r="C20" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D20" s="94" t="n">
+      <c r="D20" s="96" t="n">
         <v>3</v>
       </c>
-      <c r="E20" s="110" t="str">
+      <c r="E20" s="112" t="str">
         <v>Kho mẫu B</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -2295,18 +2306,18 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="27" customHeight="1">
-      <c r="A21" s="30" t="str"/>
-      <c r="B21" s="14" t="str">
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="31" t="str"/>
+      <c r="B21" s="15" t="str">
         <v>Cải ngọt</v>
       </c>
-      <c r="C21" s="15" t="str">
+      <c r="C21" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D21" s="94" t="n">
+      <c r="D21" s="96" t="n">
         <v>7</v>
       </c>
-      <c r="E21" s="110" t="str">
+      <c r="E21" s="112" t="str">
         <v>Kho mẫu C</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -2360,18 +2371,18 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="27" customHeight="1">
-      <c r="A22" s="30" t="str"/>
-      <c r="B22" s="14" t="str">
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="31" t="str"/>
+      <c r="B22" s="15" t="str">
         <v>Rau mẫu</v>
       </c>
-      <c r="C22" s="15" t="str">
+      <c r="C22" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D22" s="80" t="n">
+      <c r="D22" s="82" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E22" s="110" t="str">
+      <c r="E22" s="112" t="str">
         <v>Kho mẫu C</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -2425,20 +2436,20 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="72" customHeight="1">
-      <c r="A23" s="28" t="str">
+    <row r="23" ht="44" customHeight="1">
+      <c r="A23" s="29" t="str">
         <v>Trường mẫu C</v>
       </c>
-      <c r="B23" s="18" t="str">
+      <c r="B23" s="19" t="str">
         <v>Rau củ mô phỏng theo quy cách bếp mẫu</v>
       </c>
-      <c r="C23" s="19" t="str">
+      <c r="C23" s="20" t="str">
         <v>Kg</v>
       </c>
-      <c r="D23" s="88" t="n">
+      <c r="D23" s="90" t="n">
         <v>123456789.1</v>
       </c>
-      <c r="E23" s="106" t="str">
+      <c r="E23" s="108" t="str">
         <v>Kho mẫu phía đông</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -2492,18 +2503,18 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="27" customHeight="1">
-      <c r="A24" s="30" t="str"/>
-      <c r="B24" s="14" t="str">
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="31" t="str"/>
+      <c r="B24" s="15" t="str">
         <v>Tỏi</v>
       </c>
-      <c r="C24" s="15" t="str">
+      <c r="C24" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D24" s="80" t="n">
+      <c r="D24" s="82" t="n">
         <v>1234567890.1</v>
       </c>
-      <c r="E24" s="110" t="str">
+      <c r="E24" s="112" t="str">
         <v>Kho mẫu D</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2557,18 +2568,18 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="72" customHeight="1">
-      <c r="A25" s="30" t="str"/>
-      <c r="B25" s="14" t="str">
+    <row r="25" ht="44" customHeight="1">
+      <c r="A25" s="31" t="str"/>
+      <c r="B25" s="15" t="str">
         <v>Ớt mẫu</v>
       </c>
-      <c r="C25" s="15" t="str">
+      <c r="C25" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D25" s="94" t="n">
+      <c r="D25" s="96" t="n">
         <v>3</v>
       </c>
-      <c r="E25" s="110" t="str">
+      <c r="E25" s="112" t="str">
         <v>Cơ sở thực phẩm giả lập A</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -2622,1377 +2633,1377 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="72" customHeight="1">
-      <c r="A26" s="28" t="inlineStr">
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="31" t="str"/>
+      <c r="B26" s="15" t="str">
+        <v>Cải ngọt</v>
+      </c>
+      <c r="C26" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D26" s="96" t="n">
+        <v>7</v>
+      </c>
+      <c r="E26" s="112" t="str">
+        <v>Kho mẫu C</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000003ff</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007e7</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000193</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="31" t="str"/>
+      <c r="B27" s="15" t="str">
+        <v>Rau mẫu</v>
+      </c>
+      <c r="C27" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D27" s="82" t="n">
+        <v>1.234567</v>
+      </c>
+      <c r="E27" s="112" t="str">
+        <v>Kho mẫu C</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000400</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007e8</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000194</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>1.234567</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="44" customHeight="1">
+      <c r="A28" s="29" t="inlineStr">
         <is>
           <t>Trường mẫu C (tiếp)</t>
         </is>
       </c>
-      <c r="B26" s="14" t="str">
-        <v>Cải ngọt</v>
-      </c>
-      <c r="C26" s="15" t="str">
+      <c r="B28" s="15" t="str">
+        <v>Hành lá</v>
+      </c>
+      <c r="C28" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D26" s="94" t="n">
+      <c r="D28" s="82" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E28" s="112" t="str">
+        <v>Kho mẫu E</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000401</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007e9</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000195</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="31" t="str"/>
+      <c r="B29" s="15" t="str">
+        <v>Gạo tẻ</v>
+      </c>
+      <c r="C29" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D29" s="96" t="n">
+        <v>25</v>
+      </c>
+      <c r="E29" s="112" t="str">
+        <v>Kho mẫu D</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000402</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007ea</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000196</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1">
+      <c r="A30" s="31" t="str"/>
+      <c r="B30" s="15" t="str">
+        <v>Thịt heo nạc</v>
+      </c>
+      <c r="C30" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D30" s="82" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E30" s="112" t="str"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000403</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007eb</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000197</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>12.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="31" t="str"/>
+      <c r="B31" s="15" t="str">
+        <v>Trứng gà</v>
+      </c>
+      <c r="C31" s="16" t="str">
+        <v>Quả</v>
+      </c>
+      <c r="D31" s="96" t="n">
+        <v>60</v>
+      </c>
+      <c r="E31" s="112" t="str">
+        <v>Kho mẫu C</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000404</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007ec</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000198</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012e</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="31" t="str"/>
+      <c r="B32" s="15" t="str">
+        <v>Dầu ăn</v>
+      </c>
+      <c r="C32" s="16" t="str">
+        <v>Lít</v>
+      </c>
+      <c r="D32" s="82" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E32" s="112" t="str">
+        <v>Kho mẫu E</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000405</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007ed</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000199</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012f</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="31" t="str"/>
+      <c r="B33" s="15" t="str">
+        <v>Muối</v>
+      </c>
+      <c r="C33" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D33" s="82" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E33" s="112" t="str">
+        <v>Kho mẫu A</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000406</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007ee</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000019a</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="31" t="str"/>
+      <c r="B34" s="15" t="str">
+        <v>Nước mắm</v>
+      </c>
+      <c r="C34" s="16" t="str">
+        <v>Lít</v>
+      </c>
+      <c r="D34" s="96" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="112" t="str"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000407</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007ef</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000019b</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012f</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="31" t="str"/>
+      <c r="B35" s="15" t="str">
+        <v>Rau ngót</v>
+      </c>
+      <c r="C35" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D35" s="82" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E35" s="112" t="str">
+        <v>Kho mẫu B</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000408</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007f0</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000019c</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="31" t="str"/>
+      <c r="B36" s="15" t="str">
+        <v>Bí đỏ</v>
+      </c>
+      <c r="C36" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D36" s="96" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="112" t="str">
+        <v>Kho mẫu C</v>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000409</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007f1</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000019d</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="31" t="str"/>
+      <c r="B37" s="15" t="str">
+        <v>Khoai tây</v>
+      </c>
+      <c r="C37" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D37" s="96" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" s="112" t="str">
+        <v>Kho mẫu E</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000040a</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007f2</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000019e</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="31" t="str"/>
+      <c r="B38" s="15" t="str">
+        <v>Cà chua</v>
+      </c>
+      <c r="C38" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D38" s="96" t="n">
         <v>7</v>
       </c>
-      <c r="E26" s="110" t="str">
+      <c r="E38" s="112" t="str"/>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000040b</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007f3</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000019f</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="31" t="str"/>
+      <c r="B39" s="15" t="str">
+        <v>Cần ta</v>
+      </c>
+      <c r="C39" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D39" s="96" t="n">
+        <v>31</v>
+      </c>
+      <c r="E39" s="112" t="str">
+        <v>Kho mẫu D</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000040c</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007f4</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000001a0</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="31" t="str"/>
+      <c r="B40" s="15" t="str">
+        <v>Dưa leo</v>
+      </c>
+      <c r="C40" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D40" s="82" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E40" s="112" t="str">
+        <v>Kho mẫu B</v>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000040d</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007f5</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000001a1</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="31" t="str"/>
+      <c r="B41" s="15" t="str">
+        <v>Bắp cải</v>
+      </c>
+      <c r="C41" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D41" s="96" t="n">
+        <v>25</v>
+      </c>
+      <c r="E41" s="112" t="str">
         <v>Kho mẫu C</v>
       </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000003ff</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007e7</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000040e</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007f6</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000000082</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="L41" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-0000000000e6</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000193</t>
-        </is>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000001a2</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-00000000012d</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="27" customHeight="1">
-      <c r="A27" s="30" t="str"/>
-      <c r="B27" s="14" t="str">
-        <v>Rau mẫu</v>
-      </c>
-      <c r="C27" s="15" t="str">
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="31" t="str"/>
+      <c r="B42" s="15" t="str">
+        <v>Đậu cô ve</v>
+      </c>
+      <c r="C42" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D27" s="80" t="n">
-        <v>1.234567</v>
-      </c>
-      <c r="E27" s="110" t="str">
-        <v>Kho mẫu C</v>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000400</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007e8</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="D42" s="82" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E42" s="112" t="str"/>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000040f</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007f7</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="J42" s="2" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000000082</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-0000000000e6</t>
         </is>
       </c>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000194</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000001a3</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-00000000012d</t>
         </is>
       </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>1.234567</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="27" customHeight="1">
-      <c r="A28" s="30" t="str"/>
-      <c r="B28" s="14" t="str">
-        <v>Hành lá</v>
-      </c>
-      <c r="C28" s="15" t="str">
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>12.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="31" t="str"/>
+      <c r="B43" s="15" t="str">
+        <v>Su su</v>
+      </c>
+      <c r="C43" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D28" s="80" t="n">
+      <c r="D43" s="96" t="n">
+        <v>60</v>
+      </c>
+      <c r="E43" s="112" t="str">
+        <v>Kho mẫu A</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000410</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007f8</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000001a4</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="28" customHeight="1">
+      <c r="A44" s="31" t="str"/>
+      <c r="B44" s="15" t="str">
+        <v>Củ cải trắng</v>
+      </c>
+      <c r="C44" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D44" s="82" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E44" s="112" t="str">
+        <v>Kho mẫu D</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000411</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007f9</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000082</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000e6</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000001a5</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="31" t="str"/>
+      <c r="B45" s="15" t="str">
+        <v>Nấm rơm</v>
+      </c>
+      <c r="C45" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D45" s="82" t="n">
         <v>0.5</v>
       </c>
-      <c r="E28" s="110" t="str">
-        <v>Kho mẫu E</v>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000401</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007e9</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="E45" s="112" t="str">
+        <v>Kho mẫu B</v>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000412</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007fa</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000000082</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="L45" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-0000000000e6</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000195</t>
-        </is>
-      </c>
-      <c r="N28" s="2" t="inlineStr">
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000001a6</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-00000000012d</t>
         </is>
       </c>
-      <c r="O28" s="2" t="inlineStr">
+      <c r="O45" s="2" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="27" customHeight="1">
-      <c r="A29" s="30" t="str"/>
-      <c r="B29" s="14" t="str">
-        <v>Gạo tẻ</v>
-      </c>
-      <c r="C29" s="15" t="str">
+    <row r="46" ht="28" customHeight="1">
+      <c r="A46" s="31" t="str"/>
+      <c r="B46" s="15" t="str">
+        <v>Sữa chua ăn</v>
+      </c>
+      <c r="C46" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D29" s="94" t="n">
-        <v>25</v>
-      </c>
-      <c r="E29" s="110" t="str">
-        <v>Kho mẫu D</v>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000402</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007ea</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="D46" s="82" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E46" s="112" t="str"/>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000413</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000007fb</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="K46" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-000000000082</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="L46" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-0000000000e6</t>
         </is>
       </c>
-      <c r="M29" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000196</t>
-        </is>
-      </c>
-      <c r="N29" s="2" t="inlineStr">
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000001a7</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-00000000012d</t>
         </is>
       </c>
-      <c r="O29" s="2" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="27" customHeight="1">
-      <c r="A30" s="30" t="str"/>
-      <c r="B30" s="14" t="str">
-        <v>Thịt heo nạc</v>
-      </c>
-      <c r="C30" s="15" t="str">
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="28" customHeight="1">
+      <c r="A47" s="33" t="str"/>
+      <c r="B47" s="25" t="str">
+        <v>Thịt gà phi lê</v>
+      </c>
+      <c r="C47" s="26" t="str">
         <v>Kg</v>
       </c>
-      <c r="D30" s="80" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="E30" s="110" t="str"/>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000403</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007eb</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000197</t>
-        </is>
-      </c>
-      <c r="N30" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>12.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="27" customHeight="1">
-      <c r="A31" s="30" t="str"/>
-      <c r="B31" s="14" t="str">
-        <v>Trứng gà</v>
-      </c>
-      <c r="C31" s="15" t="str">
-        <v>Quả</v>
-      </c>
-      <c r="D31" s="94" t="n">
-        <v>60</v>
-      </c>
-      <c r="E31" s="110" t="str">
-        <v>Kho mẫu C</v>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000404</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007ec</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000198</t>
-        </is>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012e</t>
-        </is>
-      </c>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="27" customHeight="1">
-      <c r="A32" s="30" t="str"/>
-      <c r="B32" s="14" t="str">
-        <v>Dầu ăn</v>
-      </c>
-      <c r="C32" s="15" t="str">
-        <v>Lít</v>
-      </c>
-      <c r="D32" s="80" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E32" s="110" t="str">
-        <v>Kho mẫu E</v>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000405</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007ed</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000199</t>
-        </is>
-      </c>
-      <c r="N32" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012f</t>
-        </is>
-      </c>
-      <c r="O32" s="2" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="27" customHeight="1">
-      <c r="A33" s="30" t="str"/>
-      <c r="B33" s="14" t="str">
-        <v>Muối</v>
-      </c>
-      <c r="C33" s="15" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D33" s="80" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E33" s="110" t="str">
-        <v>Kho mẫu A</v>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000406</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007ee</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000019a</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O33" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="27" customHeight="1">
-      <c r="A34" s="30" t="str"/>
-      <c r="B34" s="14" t="str">
-        <v>Nước mắm</v>
-      </c>
-      <c r="C34" s="15" t="str">
-        <v>Lít</v>
-      </c>
-      <c r="D34" s="94" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="110" t="str"/>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000407</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007ef</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000019b</t>
-        </is>
-      </c>
-      <c r="N34" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012f</t>
-        </is>
-      </c>
-      <c r="O34" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="27" customHeight="1">
-      <c r="A35" s="30" t="str"/>
-      <c r="B35" s="14" t="str">
-        <v>Rau ngót</v>
-      </c>
-      <c r="C35" s="15" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D35" s="80" t="n">
+      <c r="D47" s="102" t="n">
         <v>0.2</v>
       </c>
-      <c r="E35" s="110" t="str">
-        <v>Kho mẫu B</v>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000408</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007f0</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000019c</t>
-        </is>
-      </c>
-      <c r="N35" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O35" s="2" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="27" customHeight="1">
-      <c r="A36" s="30" t="str"/>
-      <c r="B36" s="14" t="str">
-        <v>Bí đỏ</v>
-      </c>
-      <c r="C36" s="15" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D36" s="94" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" s="110" t="str">
-        <v>Kho mẫu C</v>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000409</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007f1</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000019d</t>
-        </is>
-      </c>
-      <c r="N36" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O36" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="27" customHeight="1">
-      <c r="A37" s="30" t="str"/>
-      <c r="B37" s="14" t="str">
-        <v>Khoai tây</v>
-      </c>
-      <c r="C37" s="15" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D37" s="94" t="n">
-        <v>3</v>
-      </c>
-      <c r="E37" s="110" t="str">
-        <v>Kho mẫu E</v>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000040a</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007f2</t>
-        </is>
-      </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M37" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000019e</t>
-        </is>
-      </c>
-      <c r="N37" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O37" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="27" customHeight="1">
-      <c r="A38" s="30" t="str"/>
-      <c r="B38" s="14" t="str">
-        <v>Cà chua</v>
-      </c>
-      <c r="C38" s="15" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D38" s="94" t="n">
-        <v>7</v>
-      </c>
-      <c r="E38" s="110" t="str"/>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000040b</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007f3</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M38" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000019f</t>
-        </is>
-      </c>
-      <c r="N38" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O38" s="2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="27" customHeight="1">
-      <c r="A39" s="30" t="str"/>
-      <c r="B39" s="14" t="str">
-        <v>Cần ta</v>
-      </c>
-      <c r="C39" s="15" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D39" s="94" t="n">
-        <v>31</v>
-      </c>
-      <c r="E39" s="110" t="str">
-        <v>Kho mẫu D</v>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000040c</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007f4</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L39" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M39" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000001a0</t>
-        </is>
-      </c>
-      <c r="N39" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O39" s="2" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="27" customHeight="1">
-      <c r="A40" s="30" t="str"/>
-      <c r="B40" s="14" t="str">
-        <v>Dưa leo</v>
-      </c>
-      <c r="C40" s="15" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D40" s="80" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E40" s="110" t="str">
-        <v>Kho mẫu B</v>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000040d</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007f5</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M40" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000001a1</t>
-        </is>
-      </c>
-      <c r="N40" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O40" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="27" customHeight="1">
-      <c r="A41" s="30" t="str"/>
-      <c r="B41" s="14" t="str">
-        <v>Bắp cải</v>
-      </c>
-      <c r="C41" s="15" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D41" s="94" t="n">
-        <v>25</v>
-      </c>
-      <c r="E41" s="110" t="str">
-        <v>Kho mẫu C</v>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000040e</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007f6</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L41" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M41" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000001a2</t>
-        </is>
-      </c>
-      <c r="N41" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O41" s="2" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="27" customHeight="1">
-      <c r="A42" s="30" t="str"/>
-      <c r="B42" s="14" t="str">
-        <v>Đậu cô ve</v>
-      </c>
-      <c r="C42" s="15" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D42" s="80" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="E42" s="110" t="str"/>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000040f</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007f7</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M42" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000001a3</t>
-        </is>
-      </c>
-      <c r="N42" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O42" s="2" t="inlineStr">
-        <is>
-          <t>12.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="27" customHeight="1">
-      <c r="A43" s="30" t="str"/>
-      <c r="B43" s="14" t="str">
-        <v>Su su</v>
-      </c>
-      <c r="C43" s="15" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D43" s="94" t="n">
-        <v>60</v>
-      </c>
-      <c r="E43" s="110" t="str">
-        <v>Kho mẫu A</v>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000410</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007f8</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K43" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L43" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M43" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000001a4</t>
-        </is>
-      </c>
-      <c r="N43" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O43" s="2" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="27" customHeight="1">
-      <c r="A44" s="30" t="str"/>
-      <c r="B44" s="14" t="str">
-        <v>Củ cải trắng</v>
-      </c>
-      <c r="C44" s="15" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D44" s="80" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E44" s="110" t="str">
-        <v>Kho mẫu D</v>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000411</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007f9</t>
-        </is>
-      </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L44" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M44" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000001a5</t>
-        </is>
-      </c>
-      <c r="N44" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O44" s="2" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="27" customHeight="1">
-      <c r="A45" s="30" t="str"/>
-      <c r="B45" s="14" t="str">
-        <v>Nấm rơm</v>
-      </c>
-      <c r="C45" s="15" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D45" s="80" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E45" s="110" t="str">
-        <v>Kho mẫu B</v>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000412</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007fa</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M45" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000001a6</t>
-        </is>
-      </c>
-      <c r="N45" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O45" s="2" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="27" customHeight="1">
-      <c r="A46" s="30" t="str"/>
-      <c r="B46" s="14" t="str">
-        <v>Sữa chua ăn</v>
-      </c>
-      <c r="C46" s="15" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D46" s="80" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E46" s="110" t="str"/>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000413</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000007fb</t>
-        </is>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000082</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000000e6</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000001a7</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O46" s="2" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="27" customHeight="1">
-      <c r="A47" s="32" t="str"/>
-      <c r="B47" s="24" t="str">
-        <v>Thịt gà phi lê</v>
-      </c>
-      <c r="C47" s="25" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D47" s="100" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E47" s="114" t="str">
+      <c r="E47" s="116" t="str">
         <v>Kho mẫu E</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -4053,12 +4064,12 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.2" right="0.2" top="0.25" bottom="0.25" header="0.12" footer="0.12"/>
-  <pageSetup paperSize="9" orientation="portrait" scale="95"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="96"/>
   <headerFooter>
     <oddFooter>&amp;RTrang &amp;P / &amp;N</oddFooter>
   </headerFooter>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="25" min="0" max="16383" man="1"/>
+    <brk id="27" min="0" max="16383" man="1"/>
   </rowBreaks>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -4073,11 +4084,11 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="33" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="7" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="19" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="6" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="15" hidden="0" customWidth="1"/>
     <col min="6" max="15" width="1" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
@@ -4118,19 +4129,19 @@
       <c r="O2" s="2"/>
     </row>
     <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="42" t="str">
+      <c r="A3" s="43" t="str">
         <v>TRƯỜNG</v>
       </c>
-      <c r="B3" s="43" t="str">
+      <c r="B3" s="44" t="str">
         <v>THÀNH PHẦN</v>
       </c>
       <c r="C3" s="145" t="str">
         <v>ĐVT</v>
       </c>
-      <c r="D3" s="43" t="str">
+      <c r="D3" s="44" t="str">
         <v>SỐ LƯỢNG</v>
       </c>
-      <c r="E3" s="44" t="str">
+      <c r="E3" s="45" t="str">
         <v>GHI CHÚ</v>
       </c>
       <c r="F3" s="2" t="str">
@@ -4164,20 +4175,20 @@
         <v>__exported_quantity</v>
       </c>
     </row>
-    <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="28" t="str">
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="29" t="str">
         <v>Trường mẫu B</v>
       </c>
-      <c r="B4" s="18" t="str">
+      <c r="B4" s="19" t="str">
         <v>Ớt hiểm đỏ</v>
       </c>
-      <c r="C4" s="19" t="str">
+      <c r="C4" s="20" t="str">
         <v>Kg</v>
       </c>
-      <c r="D4" s="88" t="n">
+      <c r="D4" s="90" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="106" t="str">
+      <c r="E4" s="108" t="str">
         <v>Kho mẫu A</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -4231,18 +4242,18 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="27" customHeight="1">
-      <c r="A5" s="30" t="str"/>
-      <c r="B5" s="14" t="str">
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="31" t="str"/>
+      <c r="B5" s="15" t="str">
         <v>Tỏi</v>
       </c>
-      <c r="C5" s="15" t="str">
+      <c r="C5" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D5" s="94" t="n">
+      <c r="D5" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="110" t="str">
+      <c r="E5" s="112" t="str">
         <v>Kho mẫu D</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4296,18 +4307,18 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="27" customHeight="1">
-      <c r="A6" s="30" t="str"/>
-      <c r="B6" s="14" t="str">
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="31" t="str"/>
+      <c r="B6" s="15" t="str">
         <v>Cà rốt</v>
       </c>
-      <c r="C6" s="15" t="str">
+      <c r="C6" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D6" s="94" t="n">
+      <c r="D6" s="96" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="110" t="str">
+      <c r="E6" s="112" t="str">
         <v>Kho mẫu B</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -4361,18 +4372,18 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="27" customHeight="1">
-      <c r="A7" s="30" t="str"/>
-      <c r="B7" s="14" t="str">
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="31" t="str"/>
+      <c r="B7" s="15" t="str">
         <v>Cải ngọt</v>
       </c>
-      <c r="C7" s="15" t="str">
+      <c r="C7" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D7" s="94" t="n">
+      <c r="D7" s="96" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="110" t="str">
+      <c r="E7" s="112" t="str">
         <v>Kho mẫu C</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -4426,18 +4437,18 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="27" customHeight="1">
-      <c r="A8" s="30" t="str"/>
-      <c r="B8" s="14" t="str">
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="31" t="str"/>
+      <c r="B8" s="15" t="str">
         <v>Rau mẫu</v>
       </c>
-      <c r="C8" s="15" t="str">
+      <c r="C8" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D8" s="80" t="n">
+      <c r="D8" s="82" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E8" s="110" t="str">
+      <c r="E8" s="112" t="str">
         <v>Kho mẫu C</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -4491,20 +4502,20 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="72" customHeight="1">
-      <c r="A9" s="28" t="str">
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="29" t="str">
         <v>Trường mẫu C</v>
       </c>
-      <c r="B9" s="18" t="str">
+      <c r="B9" s="19" t="str">
         <v>Rau củ mô phỏng sơ chế theo quy cách bếp số mười</v>
       </c>
-      <c r="C9" s="19" t="str">
+      <c r="C9" s="20" t="str">
         <v>Kg</v>
       </c>
-      <c r="D9" s="88" t="n">
+      <c r="D9" s="90" t="n">
         <v>0.2</v>
       </c>
-      <c r="E9" s="106" t="str">
+      <c r="E9" s="108" t="str">
         <v>Kho</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -4558,18 +4569,18 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="27" customHeight="1">
-      <c r="A10" s="30" t="str"/>
-      <c r="B10" s="14" t="str">
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="31" t="str"/>
+      <c r="B10" s="15" t="str">
         <v>Tỏi</v>
       </c>
-      <c r="C10" s="15" t="str">
+      <c r="C10" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D10" s="94" t="n">
+      <c r="D10" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="110" t="str">
+      <c r="E10" s="112" t="str">
         <v>Kho mẫu D</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -4623,18 +4634,18 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="27" customHeight="1">
-      <c r="A11" s="30" t="str"/>
-      <c r="B11" s="14" t="str">
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="31" t="str"/>
+      <c r="B11" s="15" t="str">
         <v>Cà rốt</v>
       </c>
-      <c r="C11" s="15" t="str">
+      <c r="C11" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D11" s="94" t="n">
+      <c r="D11" s="96" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="110" t="str">
+      <c r="E11" s="112" t="str">
         <v>Kho mẫu B</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -4688,18 +4699,18 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="27" customHeight="1">
-      <c r="A12" s="30" t="str"/>
-      <c r="B12" s="14" t="str">
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="31" t="str"/>
+      <c r="B12" s="15" t="str">
         <v>Cải ngọt</v>
       </c>
-      <c r="C12" s="15" t="str">
+      <c r="C12" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D12" s="94" t="n">
+      <c r="D12" s="96" t="n">
         <v>7</v>
       </c>
-      <c r="E12" s="110" t="str">
+      <c r="E12" s="112" t="str">
         <v>Kho mẫu C</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -4753,18 +4764,18 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="27" customHeight="1">
-      <c r="A13" s="30" t="str"/>
-      <c r="B13" s="14" t="str">
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="31" t="str"/>
+      <c r="B13" s="15" t="str">
         <v>Rau mẫu</v>
       </c>
-      <c r="C13" s="15" t="str">
+      <c r="C13" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D13" s="80" t="n">
+      <c r="D13" s="82" t="n">
         <v>1.234567</v>
       </c>
-      <c r="E13" s="110" t="str">
+      <c r="E13" s="112" t="str">
         <v>Kho mẫu C</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -4818,18 +4829,18 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="27" customHeight="1">
-      <c r="A14" s="30" t="str"/>
-      <c r="B14" s="14" t="str">
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="31" t="str"/>
+      <c r="B14" s="15" t="str">
         <v>Hành lá</v>
       </c>
-      <c r="C14" s="15" t="str">
+      <c r="C14" s="16" t="str">
         <v>Kg</v>
       </c>
-      <c r="D14" s="80" t="n">
+      <c r="D14" s="82" t="n">
         <v>0.5</v>
       </c>
-      <c r="E14" s="110" t="str">
+      <c r="E14" s="112" t="str">
         <v>Kho mẫu E</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -4883,18 +4894,18 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="27" customHeight="1">
-      <c r="A15" s="32" t="str"/>
-      <c r="B15" s="24" t="str">
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="33" t="str"/>
+      <c r="B15" s="25" t="str">
         <v>Gạo tẻ</v>
       </c>
-      <c r="C15" s="25" t="str">
+      <c r="C15" s="26" t="str">
         <v>Kg</v>
       </c>
-      <c r="D15" s="138" t="n">
+      <c r="D15" s="140" t="n">
         <v>25</v>
       </c>
-      <c r="E15" s="114" t="str">
+      <c r="E15" s="116" t="str">
         <v>Kho mẫu D</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -4955,7 +4966,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.2" right="0.2" top="0.25" bottom="0.25" header="0.12" footer="0.12"/>
-  <pageSetup paperSize="9" orientation="portrait" scale="95"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="96"/>
   <headerFooter>
     <oddFooter>&amp;RTrang &amp;P / &amp;N</oddFooter>
   </headerFooter>
@@ -4973,11 +4984,11 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="33" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="7" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="19" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="6" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="15" hidden="0" customWidth="1"/>
     <col min="6" max="15" width="1" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
@@ -5018,19 +5029,19 @@
       <c r="O2" s="2"/>
     </row>
     <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="42" t="str">
+      <c r="A3" s="43" t="str">
         <v>TRƯỜNG</v>
       </c>
-      <c r="B3" s="43" t="str">
+      <c r="B3" s="44" t="str">
         <v>THÀNH PHẦN</v>
       </c>
       <c r="C3" s="146" t="str">
         <v>ĐVT</v>
       </c>
-      <c r="D3" s="43" t="str">
+      <c r="D3" s="44" t="str">
         <v>SỐ LƯỢNG</v>
       </c>
-      <c r="E3" s="44" t="str">
+      <c r="E3" s="45" t="str">
         <v>GHI CHÚ</v>
       </c>
       <c r="F3" s="2" t="str">
@@ -5064,189 +5075,185 @@
         <v>__exported_quantity</v>
       </c>
     </row>
-    <row r="4" ht="168" customHeight="1">
-      <c r="A4" s="28" t="str">
-        <v>Trường mẫu khu vực phía đông bắc
-Điểm giao: Bếp mô phỏng khu vực phía đông A</v>
-      </c>
-      <c r="B4" s="18" t="str">
-        <v>Rau</v>
-      </c>
-      <c r="C4" s="19" t="str">
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="29" t="str">
+        <v>Trường mẫu khu vực phía đông bắc</v>
+      </c>
+      <c r="B4" s="19" t="str">
+        <v>Ớt hiểm đỏ</v>
+      </c>
+      <c r="C4" s="20" t="str">
         <v>Kg</v>
       </c>
-      <c r="D4" s="140" t="n">
+      <c r="D4" s="90" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E4" s="108" t="str">
+        <v>Kho mẫu A</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000421</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000809</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000008c</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000f0</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000190</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="31" t="str"/>
+      <c r="B5" s="15" t="str">
+        <v>Tỏi</v>
+      </c>
+      <c r="C5" s="16" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D5" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="106" t="str">
-        <v>Kho</v>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000421</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000809</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="E5" s="112" t="str">
+        <v>Kho mẫu D</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000422</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000080a</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000bf2</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000008c</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-0000000000f0</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000191</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000012d</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="33" t="str"/>
+      <c r="B6" s="25" t="str">
+        <v>Cà rốt</v>
+      </c>
+      <c r="C6" s="26" t="str">
+        <v>Kg</v>
+      </c>
+      <c r="D6" s="140" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="116" t="str">
+        <v>Kho mẫu B</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000002328</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-000000000423</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>00000000-0000-0000-0000-00000000080b</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>2026-04-22</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-00000000008c</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>00000000-0000-0000-0000-0000000000f0</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000002bf</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="168" customHeight="1">
-      <c r="A5" s="28" t="str">
-        <v>Trường mẫu khu vực phía đông bắc
-Điểm giao: Bếp mẫu B</v>
-      </c>
-      <c r="B5" s="18" t="str">
-        <v>Tỏi</v>
-      </c>
-      <c r="C5" s="19" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D5" s="140" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="106" t="str">
-        <v>Kho mẫu D</v>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000422</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000080a</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000bf2</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-22</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000008c</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000003ac</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000191</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000012d</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="27" customHeight="1">
-      <c r="A6" s="32" t="str"/>
-      <c r="B6" s="24" t="str">
-        <v>Cà rốt</v>
-      </c>
-      <c r="C6" s="25" t="str">
-        <v>Kg</v>
-      </c>
-      <c r="D6" s="138" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" s="114" t="str">
-        <v>Kho mẫu B</v>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000002328</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-000000000423</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000080b</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-22</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-00000000008c</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>00000000-0000-0000-0000-0000000003ac</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -5272,7 +5279,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.2" right="0.2" top="0.25" bottom="0.25" header="0.12" footer="0.12"/>
-  <pageSetup paperSize="9" orientation="portrait" scale="95"/>
+  <pageSetup paperSize="9" orientation="portrait" scale="96"/>
   <headerFooter>
     <oddFooter>&amp;RTrang &amp;P / &amp;N</oddFooter>
   </headerFooter>

</xml_diff>